<commit_message>
feat(insight): refactor ListenModule to dynamic insight sandbox and add dify generator integration
</commit_message>
<xml_diff>
--- a/服务及对应的dify文件.xlsx
+++ b/服务及对应的dify文件.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cursor\work\super-agent\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{738545E9-5EE2-44E2-8703-D8158F224B7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DEA82D1-248E-44FC-8AF9-7F65350AE6A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" activeTab="1" xr2:uid="{869B5D85-7F33-4AEA-A1C3-C855F7D15279}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="120">
   <si>
     <t>mychat_memory_kb</t>
   </si>
@@ -444,6 +444,12 @@
   <si>
     <t>Impromptu_Speech_Evaluation</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>app-PCvZEHnNFOGT6NppMqtudw60</t>
+  </si>
+  <si>
+    <t>Insight_Listen_Engine</t>
   </si>
 </sst>
 </file>
@@ -924,7 +930,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{424BE9F3-3748-4B33-B726-20721F5DB362}">
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="41.9296875" customWidth="1"/>
@@ -1276,7 +1282,7 @@
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
-      <c r="E19" s="2" t="s">
+      <c r="E19" s="3" t="s">
         <v>73</v>
       </c>
       <c r="F19" s="3" t="s">
@@ -1290,7 +1296,7 @@
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
-      <c r="E20" s="2" t="s">
+      <c r="E20" s="3" t="s">
         <v>77</v>
       </c>
       <c r="F20" s="3" t="s">
@@ -1304,7 +1310,7 @@
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
-      <c r="E21" s="2" t="s">
+      <c r="E21" s="3" t="s">
         <v>81</v>
       </c>
       <c r="F21" s="3" t="s">
@@ -1318,7 +1324,7 @@
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
-      <c r="E22" s="2" t="s">
+      <c r="E22" s="3" t="s">
         <v>85</v>
       </c>
       <c r="F22" s="3" t="s">
@@ -1332,7 +1338,7 @@
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
-      <c r="E23" s="2" t="s">
+      <c r="E23" s="3" t="s">
         <v>86</v>
       </c>
       <c r="F23" s="3" t="s">
@@ -1346,7 +1352,7 @@
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
-      <c r="E24" s="2" t="s">
+      <c r="E24" s="3" t="s">
         <v>89</v>
       </c>
       <c r="F24" s="3" t="s">
@@ -1360,14 +1366,14 @@
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
-      <c r="E25" s="2" t="s">
+      <c r="E25" s="3" t="s">
         <v>3</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A26" s="5" t="s">
         <v>96</v>
       </c>
@@ -1377,12 +1383,27 @@
       <c r="C26" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E26" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="F26" s="5" t="s">
+      <c r="F26" s="3" t="s">
         <v>95</v>
       </c>
+    </row>
+    <row r="27" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
+      <c r="E27" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+    </row>
+    <row r="30" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
+      <c r="E30" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
feat: implement high aesthetics system and update configs
</commit_message>
<xml_diff>
--- a/服务及对应的dify文件.xlsx
+++ b/服务及对应的dify文件.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cursor\work\super-agent\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DEA82D1-248E-44FC-8AF9-7F65350AE6A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C4B65C0-08FA-48E9-A03D-9F7751912F01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" activeTab="1" xr2:uid="{869B5D85-7F33-4AEA-A1C3-C855F7D15279}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="130">
   <si>
     <t>mychat_memory_kb</t>
   </si>
@@ -451,12 +451,47 @@
   <si>
     <t>Insight_Listen_Engine</t>
   </si>
+  <si>
+    <t>insgit_gen_flow</t>
+  </si>
+  <si>
+    <t>根据场景形成对应的会话内容</t>
+  </si>
+  <si>
+    <t>app-JAqFa8Lwrp6PsqgEdeIbQjLW</t>
+  </si>
+  <si>
+    <t>听</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>speak_engine.yml</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>cognitive_penetration_workflow</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>app-omz1BgU4iahW2FCVX0LbYa6i</t>
+  </si>
+  <si>
+    <t>说</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>读</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Write_Governance_Workflow</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -505,6 +540,24 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="5"/>
+      <color rgb="FF354052"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="5"/>
+      <color rgb="FF676F83"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="4"/>
+      <color rgb="FFA31515"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -543,7 +596,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -563,6 +616,15 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -930,7 +992,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{424BE9F3-3748-4B33-B726-20721F5DB362}">
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="41.9296875" customWidth="1"/>
@@ -1391,6 +1453,12 @@
       </c>
     </row>
     <row r="27" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
+      <c r="A27" t="s">
+        <v>123</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>121</v>
+      </c>
       <c r="E27" s="3" t="s">
         <v>118</v>
       </c>
@@ -1399,11 +1467,39 @@
       </c>
     </row>
     <row r="28" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
-      <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
+      <c r="A28" t="s">
+        <v>123</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A29" t="s">
+        <v>127</v>
+      </c>
+      <c r="F29" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="30" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
-      <c r="E30" s="3"/>
+      <c r="A30" t="s">
+        <v>128</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="F30" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="F31" s="9" t="s">
+        <v>129</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
feat: implement enhanced Dify workflows and integrate modular English learning UI components and services.
</commit_message>
<xml_diff>
--- a/服务及对应的dify文件.xlsx
+++ b/服务及对应的dify文件.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cursor\work\super-agent\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10E847C2-723F-4CFC-ABB6-C60E5F0E6CD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BD5A158-75D3-4D7D-8D72-C92A71EAAB3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" activeTab="1" xr2:uid="{869B5D85-7F33-4AEA-A1C3-C855F7D15279}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" xr2:uid="{869B5D85-7F33-4AEA-A1C3-C855F7D15279}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -40,17 +40,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="266">
   <si>
     <t>mychat_memory_kb</t>
-  </si>
-  <si>
-    <t>应用名称</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>api_key</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>app-TyztRkdBVX4kNUxA8dZ0frk7</t>
@@ -485,6 +477,425 @@
   </si>
   <si>
     <t>Write_Governance_Workflow</t>
+  </si>
+  <si>
+    <t>app-l4RcdCyDTzUPnY0GHlsgrUcs</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>English_Writing_Review</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>english_mastery_logic</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>english_wakeup_routine</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>app-jOUB4sarfRYumAyBzWhuGFYo</t>
+  </si>
+  <si>
+    <t>app_id</t>
+  </si>
+  <si>
+    <t>app_name</t>
+  </si>
+  <si>
+    <t>app_mode</t>
+  </si>
+  <si>
+    <t>api_key</t>
+  </si>
+  <si>
+    <t>created_time</t>
+  </si>
+  <si>
+    <t>635e0ef6-5484-4d3a-9d50-90db23fb5947</t>
+  </si>
+  <si>
+    <t>Impromptu_Speech_Exemplar</t>
+  </si>
+  <si>
+    <t>workflow</t>
+  </si>
+  <si>
+    <t>app-ADIa1cjKgxCbYegKjLcRnnnr</t>
+  </si>
+  <si>
+    <t>2026-06-0903:17:01</t>
+  </si>
+  <si>
+    <t>f4fee0a4-5dc5-43ce-8882-ec829b1da46e</t>
+  </si>
+  <si>
+    <t>materail_generate_url</t>
+  </si>
+  <si>
+    <t>advanced-chat</t>
+  </si>
+  <si>
+    <t>app-OShKY1EcVuLFkuxrpO28ZB0A</t>
+  </si>
+  <si>
+    <t>2026-06-0710:52:33</t>
+  </si>
+  <si>
+    <t>2a60d91e-5066-4af5-8fe8-90f9b324f030</t>
+  </si>
+  <si>
+    <t>completion</t>
+  </si>
+  <si>
+    <t>2026-05-1714:16:18</t>
+  </si>
+  <si>
+    <t>6c680ee9-dc12-4cb7-ad56-1efdce7ae6dd</t>
+  </si>
+  <si>
+    <t>material_structured_summary_workflow</t>
+  </si>
+  <si>
+    <t>2026-04-2715:15:34</t>
+  </si>
+  <si>
+    <t>f7b0ac42-a87b-4f4f-b78e-ca6fd1c6adfe</t>
+  </si>
+  <si>
+    <t>2026-05-1111:16:21</t>
+  </si>
+  <si>
+    <t>f7a8339a-e2a2-4048-af49-49856e6747ca</t>
+  </si>
+  <si>
+    <t>Pronunciation_Assessment_Engine</t>
+  </si>
+  <si>
+    <t>app-gfR3SBAHyXp3iKnIWyyRpmlI</t>
+  </si>
+  <si>
+    <t>2026-05-1410:04:42</t>
+  </si>
+  <si>
+    <t>33aebc30-9173-401a-bea0-62c6f6d16fe0</t>
+  </si>
+  <si>
+    <t>image2text</t>
+  </si>
+  <si>
+    <t>app-tY2iFt9pL38YnkRtEYcYkZXG</t>
+  </si>
+  <si>
+    <t>2026-05-0406:52:20</t>
+  </si>
+  <si>
+    <t>56a4d2c1-006c-4c46-95cc-7b6bedafbcff</t>
+  </si>
+  <si>
+    <t>2026-04-1604:44:10</t>
+  </si>
+  <si>
+    <t>f322654f-a48d-48ac-ac48-d1bbc2e57594</t>
+  </si>
+  <si>
+    <t>2026-05-1012:17:08</t>
+  </si>
+  <si>
+    <t>6cded490-c647-493e-bc34-478f784649bf</t>
+  </si>
+  <si>
+    <t>Impromptu_Speech_Enhanced</t>
+  </si>
+  <si>
+    <t>app-4pSG3G1X1P0wLIaK0qIsvExh</t>
+  </si>
+  <si>
+    <t>2026-05-2203:15:39</t>
+  </si>
+  <si>
+    <t>845bb27a-f65a-4521-a4d0-0323451a005e</t>
+  </si>
+  <si>
+    <t>text2image</t>
+  </si>
+  <si>
+    <t>app-P3RxMjvtrhr2rFAXqKcfGSFA</t>
+  </si>
+  <si>
+    <t>2026-05-0407:08:32</t>
+  </si>
+  <si>
+    <t>f4466e94-c6d8-4a3b-bf8b-0c592b45d646</t>
+  </si>
+  <si>
+    <t>2026-05-2310:04:31</t>
+  </si>
+  <si>
+    <t>262972e7-b867-4303-8ab8-795856cc844c</t>
+  </si>
+  <si>
+    <t>Impromptu_Speech_Evaluation</t>
+  </si>
+  <si>
+    <t>2026-05-1817:34:40</t>
+  </si>
+  <si>
+    <t>d7e31f94-faab-475c-89c7-58799f48e342</t>
+  </si>
+  <si>
+    <t>2026-05-1403:01:41</t>
+  </si>
+  <si>
+    <t>e04bdaa8-3d08-4439-ad67-de190ad9e557</t>
+  </si>
+  <si>
+    <t>app-UK9zXVRuldyCSGA71YQpoVpS</t>
+  </si>
+  <si>
+    <t>2026-05-1623:19:42</t>
+  </si>
+  <si>
+    <t>3f2add23-56a5-4e98-bd3d-4e8adb84cfb4</t>
+  </si>
+  <si>
+    <t>Impromptu_Speech_Prompter</t>
+  </si>
+  <si>
+    <t>app-YTMU9kmBawVOnv9CSOandhp3</t>
+  </si>
+  <si>
+    <t>2026-05-2203:14:19</t>
+  </si>
+  <si>
+    <t>fa82503b-444f-41e7-936d-c4f8b044a337</t>
+  </si>
+  <si>
+    <t>文治系统分析引擎(WriteGovernance)</t>
+  </si>
+  <si>
+    <t>app-xcidaY4l2ZbfVwL9llFyQXKA</t>
+  </si>
+  <si>
+    <t>2026-05-2407:43:29</t>
+  </si>
+  <si>
+    <t>11470c40-9678-42a3-83f7-85cda5f02671</t>
+  </si>
+  <si>
+    <t>English_Vocab_Engine</t>
+  </si>
+  <si>
+    <t>app-bqp3Cw7pb58rOpEfDeWof6bg</t>
+  </si>
+  <si>
+    <t>2026-05-1008:49:44</t>
+  </si>
+  <si>
+    <t>0fda700d-40d1-463e-b3d3-8726cdc01d33</t>
+  </si>
+  <si>
+    <t>Memory_Aid_Engine</t>
+  </si>
+  <si>
+    <t>app-aElSukJkmKmojPkVSk6H1mmN</t>
+  </si>
+  <si>
+    <t>2026-06-0812:05:29</t>
+  </si>
+  <si>
+    <t>8ea695f9-56d2-4d51-b722-69114ea10dc3</t>
+  </si>
+  <si>
+    <t>2026-05-1304:49:20</t>
+  </si>
+  <si>
+    <t>cf33959d-92f8-4f5a-8332-329e444919ce</t>
+  </si>
+  <si>
+    <t>image2text2</t>
+  </si>
+  <si>
+    <t>app-uCbUAvW6IzHig4AOOmbRAjOZ</t>
+  </si>
+  <si>
+    <t>2026-05-0706:27:37</t>
+  </si>
+  <si>
+    <t>1f82c19d-6bf2-4622-b38a-af4438245ee9</t>
+  </si>
+  <si>
+    <t>2026-05-1906:34:23</t>
+  </si>
+  <si>
+    <t>f76f76e0-aeee-4aee-9357-9626c45b34d9</t>
+  </si>
+  <si>
+    <t>CognitivePenetrationEngine</t>
+  </si>
+  <si>
+    <t>app-ZWGbI5uCdKFXj9B2yCD0Z86d</t>
+  </si>
+  <si>
+    <t>2026-05-2407:27:16</t>
+  </si>
+  <si>
+    <t>8d0ec4cf-384e-4a29-a628-2f7278bf843e</t>
+  </si>
+  <si>
+    <t>app-2lPI1fnTZXad15HQcF3xVZz5</t>
+  </si>
+  <si>
+    <t>2026-05-1013:10:50</t>
+  </si>
+  <si>
+    <t>3b6cf9ab-f6a6-488f-b5f6-c0edc52c3461</t>
+  </si>
+  <si>
+    <t>驭心博弈系统分析引擎(GameTheoryEngine)</t>
+  </si>
+  <si>
+    <t>app-YysFumsmeSAeJaQMobMpW24r</t>
+  </si>
+  <si>
+    <t>2026-05-2409:45:06</t>
+  </si>
+  <si>
+    <t>e6e97725-b3d6-4ae4-adb6-695027e9be62</t>
+  </si>
+  <si>
+    <t>Grammar_Polish_Engine</t>
+  </si>
+  <si>
+    <t>2026-05-1417:50:46</t>
+  </si>
+  <si>
+    <t>a7aef2c4-bdff-4404-9057-d5e53bea8073</t>
+  </si>
+  <si>
+    <t>doc_read_modiyg</t>
+  </si>
+  <si>
+    <t>app-G0wF6sc2GeDk7ZmV5l3wLtgM</t>
+  </si>
+  <si>
+    <t>2026-05-2610:57:31</t>
+  </si>
+  <si>
+    <t>d7257d88-c0c2-47d7-92dd-05d9e475ca24</t>
+  </si>
+  <si>
+    <t>listen_insett_workflow</t>
+  </si>
+  <si>
+    <t>app-NnsKzrUYKmhd89p9aC48YLzB</t>
+  </si>
+  <si>
+    <t>2026-05-2309:47:26</t>
+  </si>
+  <si>
+    <t>fff4614e-35a7-48f6-9cb7-301b9d9f3126</t>
+  </si>
+  <si>
+    <t>2026-05-1308:27:20</t>
+  </si>
+  <si>
+    <t>c3434f8f-9728-40c5-9674-4b0242be6492</t>
+  </si>
+  <si>
+    <t>power_game_matrix_workflow</t>
+  </si>
+  <si>
+    <t>2026-05-2003:27:23</t>
+  </si>
+  <si>
+    <t>e96a78a4-731f-4f96-99ea-e3ed0f9bb130</t>
+  </si>
+  <si>
+    <t>2026-05-1014:04:29</t>
+  </si>
+  <si>
+    <t>06744f55-096b-43b6-946a-4ed48f9c4902</t>
+  </si>
+  <si>
+    <t>Speak_Influence_Engine</t>
+  </si>
+  <si>
+    <t>app-33cYBQOXUKbRJkurDVGkzeUS</t>
+  </si>
+  <si>
+    <t>2026-05-2310:29:35</t>
+  </si>
+  <si>
+    <t>988b1ce3-1845-40f1-9211-f7b6668ec7ca</t>
+  </si>
+  <si>
+    <t>2026-04-1209:49:09</t>
+  </si>
+  <si>
+    <t>3cd2d0c7-8fcb-463f-8b3b-03f879af6539</t>
+  </si>
+  <si>
+    <t>2026-05-2406:52:28</t>
+  </si>
+  <si>
+    <t>23f90b60-7671-4130-b386-4b17b5fde233</t>
+  </si>
+  <si>
+    <t>AestheticEngine</t>
+  </si>
+  <si>
+    <t>app-sfzT1fsn8WkX5TnnIxq9qbY7</t>
+  </si>
+  <si>
+    <t>2026-05-2415:02:26</t>
+  </si>
+  <si>
+    <t>cae424a3-d1ae-4eeb-8cc5-44b1ebed3705</t>
+  </si>
+  <si>
+    <t>2026-04-1203:48:42</t>
+  </si>
+  <si>
+    <t>e2142556-f081-4425-9700-0d331dbb00d3</t>
+  </si>
+  <si>
+    <t>2026-05-2301:23:47</t>
+  </si>
+  <si>
+    <t>631a0c22-fe77-43ac-baa5-ec01211bc69e</t>
+  </si>
+  <si>
+    <t>2026-05-1417:20:13</t>
+  </si>
+  <si>
+    <t>aabd823b-7916-443e-a9f2-f357d09e2d69</t>
+  </si>
+  <si>
+    <t>2026-05-1213:53:00</t>
+  </si>
+  <si>
+    <t>f81c9849-0800-48cf-8e56-e03ef216378c</t>
+  </si>
+  <si>
+    <t>2026-05-1010:10:39</t>
+  </si>
+  <si>
+    <t>app-Eygg39qoniWss17wjWvLUvDb</t>
+  </si>
+  <si>
+    <t>2026-06-0216:15:22</t>
+  </si>
+  <si>
+    <t>2d23c873-d150-448e-9965-7e1d3094d9b1</t>
+  </si>
+  <si>
+    <t>2026-05-1007:25:00</t>
   </si>
 </sst>
 </file>
@@ -596,7 +1007,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -625,6 +1036,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -961,27 +1375,744 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04A2743E-2353-4A6B-83B4-BDC0B11420E9}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="18.9296875" customWidth="1"/>
     <col min="2" max="2" width="43.9296875" customWidth="1"/>
+    <col min="3" max="3" width="25.86328125" customWidth="1"/>
+    <col min="4" max="4" width="43.86328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A1" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="B1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C1" t="s">
+        <v>136</v>
+      </c>
+      <c r="D1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A2" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="B2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D2" t="s">
+        <v>142</v>
+      </c>
+      <c r="E2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A3" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="B3" t="s">
+        <v>145</v>
+      </c>
+      <c r="C3" t="s">
+        <v>146</v>
+      </c>
+      <c r="D3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E3" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A4" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="B4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A5" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="B5" t="s">
+        <v>153</v>
+      </c>
+      <c r="C5" t="s">
+        <v>141</v>
+      </c>
+      <c r="D5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E5" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A6" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="B6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6" t="s">
+        <v>141</v>
+      </c>
+      <c r="D6" t="s">
+        <v>71</v>
+      </c>
+      <c r="E6" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A7" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="B7" t="s">
+        <v>158</v>
+      </c>
+      <c r="C7" t="s">
+        <v>141</v>
+      </c>
+      <c r="D7" t="s">
+        <v>159</v>
+      </c>
+      <c r="E7" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A8" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="B8" t="s">
+        <v>162</v>
+      </c>
+      <c r="C8" t="s">
+        <v>141</v>
+      </c>
+      <c r="D8" t="s">
+        <v>163</v>
+      </c>
+      <c r="E8" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A9" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="B9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C9" t="s">
+        <v>146</v>
+      </c>
+      <c r="D9" t="s">
+        <v>84</v>
+      </c>
+      <c r="E9" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A10" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="B10" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" t="s">
+        <v>141</v>
+      </c>
+      <c r="D10" t="s">
+        <v>75</v>
+      </c>
+      <c r="E10" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A11" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="B11" t="s">
+        <v>170</v>
+      </c>
+      <c r="C11" t="s">
+        <v>141</v>
+      </c>
+      <c r="D11" t="s">
+        <v>171</v>
+      </c>
+      <c r="E11" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A12" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="B12" t="s">
+        <v>174</v>
+      </c>
+      <c r="C12" t="s">
+        <v>146</v>
+      </c>
+      <c r="D12" t="s">
+        <v>175</v>
+      </c>
+      <c r="E12" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A13" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="B13" t="s">
+        <v>118</v>
+      </c>
+      <c r="C13" t="s">
+        <v>150</v>
+      </c>
+      <c r="D13" t="s">
+        <v>120</v>
+      </c>
+      <c r="E13" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A14" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="B14" t="s">
+        <v>180</v>
+      </c>
+      <c r="C14" t="s">
+        <v>141</v>
+      </c>
+      <c r="D14" t="s">
+        <v>40</v>
+      </c>
+      <c r="E14" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A15" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="B15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C15" t="s">
+        <v>141</v>
+      </c>
+      <c r="D15" t="s">
+        <v>61</v>
+      </c>
+      <c r="E15" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A16" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="B16" t="s">
+        <v>58</v>
+      </c>
+      <c r="C16" t="s">
+        <v>150</v>
+      </c>
+      <c r="D16" t="s">
+        <v>185</v>
+      </c>
+      <c r="E16" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A17" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="B17" t="s">
+        <v>188</v>
+      </c>
+      <c r="C17" t="s">
+        <v>141</v>
+      </c>
+      <c r="D17" t="s">
+        <v>189</v>
+      </c>
+      <c r="E17" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A18" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="B18" t="s">
+        <v>192</v>
+      </c>
+      <c r="C18" t="s">
+        <v>141</v>
+      </c>
+      <c r="D18" t="s">
+        <v>193</v>
+      </c>
+      <c r="E18" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A19" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="B19" t="s">
+        <v>196</v>
+      </c>
+      <c r="C19" t="s">
+        <v>141</v>
+      </c>
+      <c r="D19" t="s">
+        <v>197</v>
+      </c>
+      <c r="E19" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A20" s="10" t="s">
+        <v>199</v>
+      </c>
+      <c r="B20" t="s">
+        <v>200</v>
+      </c>
+      <c r="C20" t="s">
+        <v>141</v>
+      </c>
+      <c r="D20" t="s">
+        <v>201</v>
+      </c>
+      <c r="E20" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A21" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="B21" t="s">
+        <v>68</v>
+      </c>
+      <c r="C21" t="s">
+        <v>141</v>
+      </c>
+      <c r="D21" t="s">
+        <v>67</v>
+      </c>
+      <c r="E21" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A22" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="B22" t="s">
+        <v>206</v>
+      </c>
+      <c r="C22" t="s">
+        <v>141</v>
+      </c>
+      <c r="D22" t="s">
+        <v>207</v>
+      </c>
+      <c r="E22" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A23" s="10" t="s">
+        <v>209</v>
+      </c>
+      <c r="B23" t="s">
+        <v>81</v>
+      </c>
+      <c r="C23" t="s">
+        <v>146</v>
+      </c>
+      <c r="D23" t="s">
+        <v>83</v>
+      </c>
+      <c r="E23" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A24" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B24" t="s">
+        <v>212</v>
+      </c>
+      <c r="C24" t="s">
+        <v>141</v>
+      </c>
+      <c r="D24" t="s">
+        <v>213</v>
+      </c>
+      <c r="E24" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A25" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="B25" t="s">
+        <v>74</v>
+      </c>
+      <c r="C25" t="s">
+        <v>141</v>
+      </c>
+      <c r="D25" t="s">
+        <v>216</v>
+      </c>
+      <c r="E25" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A26" s="10" t="s">
+        <v>218</v>
+      </c>
+      <c r="B26" t="s">
+        <v>219</v>
+      </c>
+      <c r="C26" t="s">
+        <v>141</v>
+      </c>
+      <c r="D26" t="s">
+        <v>220</v>
+      </c>
+      <c r="E26" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A27" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="B27" t="s">
+        <v>223</v>
+      </c>
+      <c r="C27" t="s">
+        <v>141</v>
+      </c>
+      <c r="D27" t="s">
+        <v>41</v>
+      </c>
+      <c r="E27" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A28" s="10" t="s">
+        <v>225</v>
+      </c>
+      <c r="B28" t="s">
+        <v>226</v>
+      </c>
+      <c r="C28" t="s">
+        <v>146</v>
+      </c>
+      <c r="D28" t="s">
+        <v>227</v>
+      </c>
+      <c r="E28" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A29" s="10" t="s">
+        <v>229</v>
+      </c>
+      <c r="B29" t="s">
+        <v>230</v>
+      </c>
+      <c r="C29" t="s">
+        <v>141</v>
+      </c>
+      <c r="D29" t="s">
+        <v>231</v>
+      </c>
+      <c r="E29" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A30" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="B30" t="s">
+        <v>66</v>
+      </c>
+      <c r="C30" t="s">
+        <v>141</v>
+      </c>
+      <c r="D30" t="s">
+        <v>64</v>
+      </c>
+      <c r="E30" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A31" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="B31" t="s">
+        <v>236</v>
+      </c>
+      <c r="C31" t="s">
+        <v>141</v>
+      </c>
+      <c r="D31" t="s">
+        <v>92</v>
+      </c>
+      <c r="E31" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A32" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="B32" t="s">
+        <v>73</v>
+      </c>
+      <c r="C32" t="s">
+        <v>141</v>
+      </c>
+      <c r="D32" t="s">
+        <v>36</v>
+      </c>
+      <c r="E32" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A33" s="10" t="s">
+        <v>240</v>
+      </c>
+      <c r="B33" t="s">
+        <v>241</v>
+      </c>
+      <c r="C33" t="s">
+        <v>141</v>
+      </c>
+      <c r="D33" t="s">
+        <v>242</v>
+      </c>
+      <c r="E33" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A34" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="B34" t="s">
+        <v>88</v>
+      </c>
+      <c r="C34" t="s">
+        <v>141</v>
+      </c>
+      <c r="D34" t="s">
+        <v>87</v>
+      </c>
+      <c r="E34" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A35" s="10" t="s">
+        <v>246</v>
+      </c>
+      <c r="B35" t="s">
+        <v>212</v>
+      </c>
+      <c r="C35" t="s">
+        <v>141</v>
+      </c>
+      <c r="D35" t="s">
+        <v>124</v>
+      </c>
+      <c r="E35" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A36" s="10" t="s">
+        <v>248</v>
+      </c>
+      <c r="B36" t="s">
+        <v>249</v>
+      </c>
+      <c r="C36" t="s">
+        <v>141</v>
+      </c>
+      <c r="D36" t="s">
+        <v>250</v>
+      </c>
+      <c r="E36" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A37" s="10" t="s">
+        <v>252</v>
+      </c>
+      <c r="B37" t="s">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>146</v>
+      </c>
+      <c r="D37" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
+      <c r="E37" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A38" s="10" t="s">
+        <v>254</v>
+      </c>
+      <c r="B38" t="s">
+        <v>117</v>
+      </c>
+      <c r="C38" t="s">
+        <v>141</v>
+      </c>
+      <c r="D38" t="s">
+        <v>116</v>
+      </c>
+      <c r="E38" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A39" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="B39" t="s">
+        <v>59</v>
+      </c>
+      <c r="C39" t="s">
+        <v>141</v>
+      </c>
+      <c r="D39" t="s">
+        <v>37</v>
+      </c>
+      <c r="E39" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A40" s="10" t="s">
+        <v>258</v>
+      </c>
+      <c r="B40" t="s">
+        <v>70</v>
+      </c>
+      <c r="C40" t="s">
+        <v>141</v>
+      </c>
+      <c r="D40" t="s">
+        <v>133</v>
+      </c>
+      <c r="E40" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A41" s="10" t="s">
+        <v>260</v>
+      </c>
+      <c r="B41" t="s">
+        <v>77</v>
+      </c>
+      <c r="C41" t="s">
+        <v>146</v>
+      </c>
+      <c r="D41" t="s">
+        <v>38</v>
+      </c>
+      <c r="E41" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A42" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="B42" t="s">
+        <v>145</v>
+      </c>
+      <c r="C42" t="s">
+        <v>146</v>
+      </c>
+      <c r="D42" t="s">
+        <v>262</v>
+      </c>
+      <c r="E42" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A43" s="10" t="s">
+        <v>264</v>
+      </c>
+      <c r="B43" t="s">
+        <v>78</v>
+      </c>
+      <c r="C43" t="s">
+        <v>141</v>
+      </c>
+      <c r="D43" t="s">
+        <v>39</v>
+      </c>
+      <c r="E43" t="s">
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -992,7 +2123,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{424BE9F3-3748-4B33-B726-20721F5DB362}">
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="41.9296875" customWidth="1"/>
@@ -1005,431 +2136,431 @@
   <sheetData>
     <row r="1" spans="1:6" ht="28.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>104</v>
-      </c>
       <c r="F1" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>105</v>
-      </c>
       <c r="F2" s="3" t="s">
-        <v>72</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>110</v>
-      </c>
       <c r="F6" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F10" s="2"/>
     </row>
     <row r="11" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>41</v>
+        <v>128</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>80</v>
+        <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="D14" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A15" s="2"/>
       <c r="B15" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A16" s="2"/>
       <c r="B16" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A17" s="2"/>
       <c r="B17" s="4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F17" s="3" t="s">
         <v>66</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A18" s="2"/>
       <c r="B18" s="4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A19" s="2"/>
       <c r="B19" s="4" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>74</v>
+        <v>131</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A20" s="2"/>
       <c r="B20" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A21" s="2"/>
       <c r="B21" s="4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A22" s="2"/>
       <c r="B22" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
       <c r="E22" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A23" s="2"/>
       <c r="B23" s="4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="E23" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="F23" s="3" t="s">
         <v>86</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A24" s="2"/>
       <c r="B24" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="3" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A25" s="2"/>
       <c r="B25" s="4" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
       <c r="E25" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>0</v>
@@ -1437,68 +2568,73 @@
     </row>
     <row r="26" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A26" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B26" t="s">
+        <v>95</v>
+      </c>
+      <c r="C26" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="B26" t="s">
-        <v>97</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>98</v>
-      </c>
       <c r="E26" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="F29" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="F30" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.4">
       <c r="F31" s="9" t="s">
-        <v>129</v>
+        <v>127</v>
+      </c>
+    </row>
+    <row r="36" spans="10:10" x14ac:dyDescent="0.4">
+      <c r="J36" t="s">
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement vocabulary server with SQLite database and RESTful API endpoints
</commit_message>
<xml_diff>
--- a/服务及对应的dify文件.xlsx
+++ b/服务及对应的dify文件.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cursor\work\super-agent\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BD5A158-75D3-4D7D-8D72-C92A71EAAB3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{288454FD-3585-45B3-BEBB-EEA4D7C63F87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" xr2:uid="{869B5D85-7F33-4AEA-A1C3-C855F7D15279}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="267">
   <si>
     <t>mychat_memory_kb</t>
   </si>
@@ -257,13 +257,7 @@
     <t>生成带有 A2-C1 难度评级、真实音频接入字段及潜台词分析的商务/政务听力语料</t>
   </si>
   <si>
-    <t>english_wakeup_routine</t>
-  </si>
-  <si>
     <t>app-cArGQg7bAnePU0ts63FoHrAG</t>
-  </si>
-  <si>
-    <t>english_mastery_logic</t>
   </si>
   <si>
     <t>English_Word_Enricher</t>
@@ -896,6 +890,18 @@
   </si>
   <si>
     <t>2026-05-1007:25:00</t>
+  </si>
+  <si>
+    <t>materail_generate_url</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>english_mastery_logic</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>english_wakeup_routine</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1386,733 +1392,733 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A1" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="B1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C1" t="s">
         <v>134</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>135</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>136</v>
-      </c>
-      <c r="D1" t="s">
-        <v>137</v>
-      </c>
-      <c r="E1" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A2" s="10" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D2" t="s">
         <v>140</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>141</v>
-      </c>
-      <c r="D2" t="s">
-        <v>142</v>
-      </c>
-      <c r="E2" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A3" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="B3" t="s">
+        <v>264</v>
+      </c>
+      <c r="C3" t="s">
         <v>144</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
         <v>145</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
         <v>146</v>
-      </c>
-      <c r="D3" t="s">
-        <v>147</v>
-      </c>
-      <c r="E3" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A4" s="10" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B4" t="s">
         <v>58</v>
       </c>
       <c r="C4" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D4" t="s">
         <v>35</v>
       </c>
       <c r="E4" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A5" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="B5" t="s">
+        <v>151</v>
+      </c>
+      <c r="C5" t="s">
+        <v>139</v>
+      </c>
+      <c r="D5" t="s">
+        <v>77</v>
+      </c>
+      <c r="E5" t="s">
         <v>152</v>
-      </c>
-      <c r="B5" t="s">
-        <v>153</v>
-      </c>
-      <c r="C5" t="s">
-        <v>141</v>
-      </c>
-      <c r="D5" t="s">
-        <v>79</v>
-      </c>
-      <c r="E5" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A6" s="10" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B6" t="s">
-        <v>72</v>
+        <v>265</v>
       </c>
       <c r="C6" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E6" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A7" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="B7" t="s">
+        <v>156</v>
+      </c>
+      <c r="C7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D7" t="s">
         <v>157</v>
       </c>
-      <c r="B7" t="s">
+      <c r="E7" t="s">
         <v>158</v>
-      </c>
-      <c r="C7" t="s">
-        <v>141</v>
-      </c>
-      <c r="D7" t="s">
-        <v>159</v>
-      </c>
-      <c r="E7" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A8" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="B8" t="s">
+        <v>160</v>
+      </c>
+      <c r="C8" t="s">
+        <v>139</v>
+      </c>
+      <c r="D8" t="s">
         <v>161</v>
       </c>
-      <c r="B8" t="s">
+      <c r="E8" t="s">
         <v>162</v>
-      </c>
-      <c r="C8" t="s">
-        <v>141</v>
-      </c>
-      <c r="D8" t="s">
-        <v>163</v>
-      </c>
-      <c r="E8" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A9" s="10" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C9" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D9" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E9" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A10" s="10" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B10" t="s">
         <v>59</v>
       </c>
       <c r="C10" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E10" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A11" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="B11" t="s">
+        <v>168</v>
+      </c>
+      <c r="C11" t="s">
+        <v>139</v>
+      </c>
+      <c r="D11" t="s">
         <v>169</v>
       </c>
-      <c r="B11" t="s">
+      <c r="E11" t="s">
         <v>170</v>
-      </c>
-      <c r="C11" t="s">
-        <v>141</v>
-      </c>
-      <c r="D11" t="s">
-        <v>171</v>
-      </c>
-      <c r="E11" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A12" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="B12" t="s">
+        <v>172</v>
+      </c>
+      <c r="C12" t="s">
+        <v>144</v>
+      </c>
+      <c r="D12" t="s">
         <v>173</v>
       </c>
-      <c r="B12" t="s">
+      <c r="E12" t="s">
         <v>174</v>
-      </c>
-      <c r="C12" t="s">
-        <v>146</v>
-      </c>
-      <c r="D12" t="s">
-        <v>175</v>
-      </c>
-      <c r="E12" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A13" s="10" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B13" t="s">
+        <v>116</v>
+      </c>
+      <c r="C13" t="s">
+        <v>148</v>
+      </c>
+      <c r="D13" t="s">
         <v>118</v>
       </c>
-      <c r="C13" t="s">
-        <v>150</v>
-      </c>
-      <c r="D13" t="s">
-        <v>120</v>
-      </c>
       <c r="E13" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A14" s="10" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C14" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D14" t="s">
         <v>40</v>
       </c>
       <c r="E14" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A15" s="10" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B15" t="s">
         <v>62</v>
       </c>
       <c r="C15" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D15" t="s">
         <v>61</v>
       </c>
       <c r="E15" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A16" s="10" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B16" t="s">
         <v>58</v>
       </c>
       <c r="C16" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D16" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="E16" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A17" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="B17" t="s">
+        <v>186</v>
+      </c>
+      <c r="C17" t="s">
+        <v>139</v>
+      </c>
+      <c r="D17" t="s">
         <v>187</v>
       </c>
-      <c r="B17" t="s">
+      <c r="E17" t="s">
         <v>188</v>
-      </c>
-      <c r="C17" t="s">
-        <v>141</v>
-      </c>
-      <c r="D17" t="s">
-        <v>189</v>
-      </c>
-      <c r="E17" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A18" s="10" t="s">
+        <v>189</v>
+      </c>
+      <c r="B18" t="s">
+        <v>190</v>
+      </c>
+      <c r="C18" t="s">
+        <v>139</v>
+      </c>
+      <c r="D18" t="s">
         <v>191</v>
       </c>
-      <c r="B18" t="s">
+      <c r="E18" t="s">
         <v>192</v>
-      </c>
-      <c r="C18" t="s">
-        <v>141</v>
-      </c>
-      <c r="D18" t="s">
-        <v>193</v>
-      </c>
-      <c r="E18" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A19" s="10" t="s">
+        <v>193</v>
+      </c>
+      <c r="B19" t="s">
+        <v>194</v>
+      </c>
+      <c r="C19" t="s">
+        <v>139</v>
+      </c>
+      <c r="D19" t="s">
         <v>195</v>
       </c>
-      <c r="B19" t="s">
+      <c r="E19" t="s">
         <v>196</v>
-      </c>
-      <c r="C19" t="s">
-        <v>141</v>
-      </c>
-      <c r="D19" t="s">
-        <v>197</v>
-      </c>
-      <c r="E19" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A20" s="10" t="s">
+        <v>197</v>
+      </c>
+      <c r="B20" t="s">
+        <v>198</v>
+      </c>
+      <c r="C20" t="s">
+        <v>139</v>
+      </c>
+      <c r="D20" t="s">
         <v>199</v>
       </c>
-      <c r="B20" t="s">
+      <c r="E20" t="s">
         <v>200</v>
-      </c>
-      <c r="C20" t="s">
-        <v>141</v>
-      </c>
-      <c r="D20" t="s">
-        <v>201</v>
-      </c>
-      <c r="E20" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A21" s="10" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B21" t="s">
         <v>68</v>
       </c>
       <c r="C21" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D21" t="s">
         <v>67</v>
       </c>
       <c r="E21" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A22" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="B22" t="s">
+        <v>204</v>
+      </c>
+      <c r="C22" t="s">
+        <v>139</v>
+      </c>
+      <c r="D22" t="s">
         <v>205</v>
       </c>
-      <c r="B22" t="s">
+      <c r="E22" t="s">
         <v>206</v>
-      </c>
-      <c r="C22" t="s">
-        <v>141</v>
-      </c>
-      <c r="D22" t="s">
-        <v>207</v>
-      </c>
-      <c r="E22" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A23" s="10" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B23" t="s">
+        <v>79</v>
+      </c>
+      <c r="C23" t="s">
+        <v>144</v>
+      </c>
+      <c r="D23" t="s">
         <v>81</v>
       </c>
-      <c r="C23" t="s">
-        <v>146</v>
-      </c>
-      <c r="D23" t="s">
-        <v>83</v>
-      </c>
       <c r="E23" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A24" s="10" t="s">
+        <v>209</v>
+      </c>
+      <c r="B24" t="s">
+        <v>210</v>
+      </c>
+      <c r="C24" t="s">
+        <v>139</v>
+      </c>
+      <c r="D24" t="s">
         <v>211</v>
       </c>
-      <c r="B24" t="s">
+      <c r="E24" t="s">
         <v>212</v>
-      </c>
-      <c r="C24" t="s">
-        <v>141</v>
-      </c>
-      <c r="D24" t="s">
-        <v>213</v>
-      </c>
-      <c r="E24" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A25" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="B25" t="s">
+        <v>72</v>
+      </c>
+      <c r="C25" t="s">
+        <v>139</v>
+      </c>
+      <c r="D25" t="s">
+        <v>214</v>
+      </c>
+      <c r="E25" t="s">
         <v>215</v>
-      </c>
-      <c r="B25" t="s">
-        <v>74</v>
-      </c>
-      <c r="C25" t="s">
-        <v>141</v>
-      </c>
-      <c r="D25" t="s">
-        <v>216</v>
-      </c>
-      <c r="E25" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A26" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="B26" t="s">
+        <v>217</v>
+      </c>
+      <c r="C26" t="s">
+        <v>139</v>
+      </c>
+      <c r="D26" t="s">
         <v>218</v>
       </c>
-      <c r="B26" t="s">
+      <c r="E26" t="s">
         <v>219</v>
-      </c>
-      <c r="C26" t="s">
-        <v>141</v>
-      </c>
-      <c r="D26" t="s">
-        <v>220</v>
-      </c>
-      <c r="E26" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A27" s="10" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B27" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C27" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D27" t="s">
         <v>41</v>
       </c>
       <c r="E27" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A28" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="B28" t="s">
+        <v>224</v>
+      </c>
+      <c r="C28" t="s">
+        <v>144</v>
+      </c>
+      <c r="D28" t="s">
         <v>225</v>
       </c>
-      <c r="B28" t="s">
+      <c r="E28" t="s">
         <v>226</v>
-      </c>
-      <c r="C28" t="s">
-        <v>146</v>
-      </c>
-      <c r="D28" t="s">
-        <v>227</v>
-      </c>
-      <c r="E28" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A29" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="B29" t="s">
+        <v>228</v>
+      </c>
+      <c r="C29" t="s">
+        <v>139</v>
+      </c>
+      <c r="D29" t="s">
         <v>229</v>
       </c>
-      <c r="B29" t="s">
+      <c r="E29" t="s">
         <v>230</v>
-      </c>
-      <c r="C29" t="s">
-        <v>141</v>
-      </c>
-      <c r="D29" t="s">
-        <v>231</v>
-      </c>
-      <c r="E29" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A30" s="10" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B30" t="s">
         <v>66</v>
       </c>
       <c r="C30" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D30" t="s">
         <v>64</v>
       </c>
       <c r="E30" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A31" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="B31" t="s">
+        <v>234</v>
+      </c>
+      <c r="C31" t="s">
+        <v>139</v>
+      </c>
+      <c r="D31" t="s">
+        <v>90</v>
+      </c>
+      <c r="E31" t="s">
         <v>235</v>
-      </c>
-      <c r="B31" t="s">
-        <v>236</v>
-      </c>
-      <c r="C31" t="s">
-        <v>141</v>
-      </c>
-      <c r="D31" t="s">
-        <v>92</v>
-      </c>
-      <c r="E31" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A32" s="10" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B32" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C32" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D32" t="s">
         <v>36</v>
       </c>
       <c r="E32" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A33" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="B33" t="s">
+        <v>239</v>
+      </c>
+      <c r="C33" t="s">
+        <v>139</v>
+      </c>
+      <c r="D33" t="s">
         <v>240</v>
       </c>
-      <c r="B33" t="s">
+      <c r="E33" t="s">
         <v>241</v>
-      </c>
-      <c r="C33" t="s">
-        <v>141</v>
-      </c>
-      <c r="D33" t="s">
-        <v>242</v>
-      </c>
-      <c r="E33" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A34" s="10" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B34" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C34" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D34" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E34" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A35" s="10" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B35" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C35" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D35" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E35" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A36" s="10" t="s">
+        <v>246</v>
+      </c>
+      <c r="B36" t="s">
+        <v>247</v>
+      </c>
+      <c r="C36" t="s">
+        <v>139</v>
+      </c>
+      <c r="D36" t="s">
         <v>248</v>
       </c>
-      <c r="B36" t="s">
+      <c r="E36" t="s">
         <v>249</v>
-      </c>
-      <c r="C36" t="s">
-        <v>141</v>
-      </c>
-      <c r="D36" t="s">
-        <v>250</v>
-      </c>
-      <c r="E36" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A37" s="10" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B37" t="s">
         <v>0</v>
       </c>
       <c r="C37" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D37" t="s">
         <v>1</v>
       </c>
       <c r="E37" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A38" s="10" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B38" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C38" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D38" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E38" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A39" s="10" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B39" t="s">
         <v>59</v>
       </c>
       <c r="C39" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D39" t="s">
         <v>37</v>
       </c>
       <c r="E39" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A40" s="10" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B40" t="s">
-        <v>70</v>
+        <v>266</v>
       </c>
       <c r="C40" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D40" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E40" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A41" s="10" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B41" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C41" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D41" t="s">
         <v>38</v>
       </c>
       <c r="E41" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A42" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="B42" t="s">
+        <v>143</v>
+      </c>
+      <c r="C42" t="s">
         <v>144</v>
       </c>
-      <c r="B42" t="s">
-        <v>145</v>
-      </c>
-      <c r="C42" t="s">
-        <v>146</v>
-      </c>
       <c r="D42" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="E42" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A43" s="10" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B43" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C43" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D43" t="s">
         <v>39</v>
       </c>
       <c r="E43" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
     </row>
   </sheetData>
@@ -2142,13 +2148,13 @@
         <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>57</v>
@@ -2162,16 +2168,16 @@
         <v>5</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>103</v>
-      </c>
       <c r="F2" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
@@ -2202,16 +2208,16 @@
         <v>9</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
@@ -2231,7 +2237,7 @@
         <v>36</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
@@ -2239,19 +2245,19 @@
         <v>12</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>108</v>
-      </c>
       <c r="F6" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
@@ -2322,7 +2328,7 @@
         <v>20</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>56</v>
@@ -2349,7 +2355,7 @@
         <v>38</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
@@ -2366,10 +2372,10 @@
         <v>48</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
@@ -2389,7 +2395,7 @@
         <v>40</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
@@ -2409,7 +2415,7 @@
         <v>41</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
@@ -2420,10 +2426,10 @@
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
@@ -2471,26 +2477,26 @@
     <row r="19" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A19" s="2"/>
       <c r="B19" s="4" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A20" s="2"/>
       <c r="B20" s="4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>59</v>
@@ -2499,63 +2505,63 @@
     <row r="21" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A21" s="2"/>
       <c r="B21" s="4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A22" s="2"/>
       <c r="B22" s="4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
       <c r="E22" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A23" s="2"/>
       <c r="B23" s="4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="E23" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="F23" s="3" t="s">
         <v>84</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A24" s="2"/>
       <c r="B24" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A25" s="2"/>
       <c r="B25" s="4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
@@ -2568,73 +2574,73 @@
     </row>
     <row r="26" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A26" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B26" t="s">
+        <v>93</v>
+      </c>
+      <c r="C26" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="B26" t="s">
-        <v>95</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>96</v>
-      </c>
       <c r="E26" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="F29" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F30" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.4">
       <c r="F31" s="9" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="36" spans="10:10" x14ac:dyDescent="0.4">
       <c r="J36" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement impromptu speech tab with voice recording, Dify API integration, and evaluation capabilities
</commit_message>
<xml_diff>
--- a/服务及对应的dify文件.xlsx
+++ b/服务及对应的dify文件.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cursor\work\super-agent\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{288454FD-3585-45B3-BEBB-EEA4D7C63F87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79EF54FF-6F6D-45DD-958D-2A9183BED0C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" xr2:uid="{869B5D85-7F33-4AEA-A1C3-C855F7D15279}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="269">
   <si>
     <t>mychat_memory_kb</t>
   </si>
@@ -903,12 +903,20 @@
     <t>english_wakeup_routine</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>listen_material_generator</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Listening_Comparison_Engine</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -975,6 +983,15 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1013,7 +1030,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1045,6 +1062,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1445,8 +1465,8 @@
       <c r="A4" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="B4" t="s">
-        <v>58</v>
+      <c r="B4" s="11" t="s">
+        <v>267</v>
       </c>
       <c r="C4" t="s">
         <v>148</v>
@@ -2040,8 +2060,8 @@
       <c r="A39" s="10" t="s">
         <v>254</v>
       </c>
-      <c r="B39" t="s">
-        <v>59</v>
+      <c r="B39" s="11" t="s">
+        <v>268</v>
       </c>
       <c r="C39" t="s">
         <v>139</v>

</xml_diff>

<commit_message>
feat: inject user current profile into dify api calls and backend routes
</commit_message>
<xml_diff>
--- a/服务及对应的dify文件.xlsx
+++ b/服务及对应的dify文件.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cursor\work\super-agent\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79EF54FF-6F6D-45DD-958D-2A9183BED0C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D25BC422-920B-438D-BD72-1CD19C55813F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" xr2:uid="{869B5D85-7F33-4AEA-A1C3-C855F7D15279}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="265">
   <si>
     <t>mychat_memory_kb</t>
   </si>
@@ -529,18 +529,9 @@
     <t>f4fee0a4-5dc5-43ce-8882-ec829b1da46e</t>
   </si>
   <si>
-    <t>materail_generate_url</t>
-  </si>
-  <si>
     <t>advanced-chat</t>
   </si>
   <si>
-    <t>app-OShKY1EcVuLFkuxrpO28ZB0A</t>
-  </si>
-  <si>
-    <t>2026-06-0710:52:33</t>
-  </si>
-  <si>
     <t>2a60d91e-5066-4af5-8fe8-90f9b324f030</t>
   </si>
   <si>
@@ -727,18 +718,9 @@
     <t>2026-05-1906:34:23</t>
   </si>
   <si>
-    <t>f76f76e0-aeee-4aee-9357-9626c45b34d9</t>
-  </si>
-  <si>
     <t>CognitivePenetrationEngine</t>
   </si>
   <si>
-    <t>app-ZWGbI5uCdKFXj9B2yCD0Z86d</t>
-  </si>
-  <si>
-    <t>2026-05-2407:27:16</t>
-  </si>
-  <si>
     <t>8d0ec4cf-384e-4a29-a628-2f7278bf843e</t>
   </si>
   <si>
@@ -814,18 +796,6 @@
     <t>2026-05-1014:04:29</t>
   </si>
   <si>
-    <t>06744f55-096b-43b6-946a-4ed48f9c4902</t>
-  </si>
-  <si>
-    <t>Speak_Influence_Engine</t>
-  </si>
-  <si>
-    <t>app-33cYBQOXUKbRJkurDVGkzeUS</t>
-  </si>
-  <si>
-    <t>2026-05-2310:29:35</t>
-  </si>
-  <si>
     <t>988b1ce3-1845-40f1-9211-f7b6668ec7ca</t>
   </si>
   <si>
@@ -892,23 +862,37 @@
     <t>2026-05-1007:25:00</t>
   </si>
   <si>
-    <t>materail_generate_url</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+    <t>d94f726d-d0fd-40a2-8997-3f85fd8ab3e2</t>
+  </si>
+  <si>
+    <t>app-F6daqhSXH942sBrnGki4kzZq</t>
+  </si>
+  <si>
+    <t>2026-06-0912:30:06</t>
   </si>
   <si>
     <t>english_mastery_logic</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>694843b2-96e0-4b36-b438-c7a1110116e8</t>
+  </si>
+  <si>
+    <t>video_subtitle_transcription_workflow</t>
+  </si>
+  <si>
+    <t>app-2LpliLyJ8viBKpacvyoOHSAV</t>
+  </si>
+  <si>
+    <t>2026-06-1008:58:18</t>
   </si>
   <si>
     <t>english_wakeup_routine</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>listen_material_generator</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Listening_Comparison_Engine</t>
+  </si>
+  <si>
+    <t>materail_generate_url_enhanced</t>
+  </si>
+  <si>
+    <t>custom_theme_extraction</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1401,7 +1385,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04A2743E-2353-4A6B-83B4-BDC0B11420E9}">
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="18.9296875" customWidth="1"/>
@@ -1429,359 +1413,359 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A2" s="10" t="s">
-        <v>137</v>
+        <v>182</v>
       </c>
       <c r="B2" t="s">
-        <v>138</v>
+        <v>183</v>
       </c>
       <c r="C2" t="s">
         <v>139</v>
       </c>
       <c r="D2" t="s">
-        <v>140</v>
+        <v>184</v>
       </c>
       <c r="E2" t="s">
-        <v>141</v>
+        <v>185</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A3" s="10" t="s">
-        <v>142</v>
-      </c>
-      <c r="B3" t="s">
-        <v>264</v>
+        <v>147</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>148</v>
       </c>
       <c r="C3" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="D3" t="s">
-        <v>145</v>
+        <v>77</v>
       </c>
       <c r="E3" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A4" s="10" t="s">
-        <v>147</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>267</v>
+        <v>152</v>
+      </c>
+      <c r="B4" t="s">
+        <v>153</v>
       </c>
       <c r="C4" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="D4" t="s">
-        <v>35</v>
+        <v>154</v>
       </c>
       <c r="E4" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A5" s="10" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="B5" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C5" t="s">
         <v>139</v>
       </c>
       <c r="D5" t="s">
-        <v>77</v>
+        <v>158</v>
       </c>
       <c r="E5" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A6" s="10" t="s">
-        <v>153</v>
+        <v>254</v>
       </c>
       <c r="B6" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C6" t="s">
         <v>139</v>
       </c>
       <c r="D6" t="s">
-        <v>70</v>
+        <v>255</v>
       </c>
       <c r="E6" t="s">
-        <v>154</v>
+        <v>256</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A7" s="10" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="B7" t="s">
-        <v>156</v>
+        <v>257</v>
       </c>
       <c r="C7" t="s">
         <v>139</v>
       </c>
       <c r="D7" t="s">
-        <v>157</v>
+        <v>70</v>
       </c>
       <c r="E7" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A8" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B8" t="s">
-        <v>160</v>
+        <v>84</v>
       </c>
       <c r="C8" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D8" t="s">
+        <v>82</v>
+      </c>
+      <c r="E8" t="s">
         <v>161</v>
-      </c>
-      <c r="E8" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A9" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="B9" t="s">
+        <v>59</v>
+      </c>
+      <c r="C9" t="s">
+        <v>139</v>
+      </c>
+      <c r="D9" t="s">
+        <v>73</v>
+      </c>
+      <c r="E9" t="s">
         <v>163</v>
-      </c>
-      <c r="B9" t="s">
-        <v>84</v>
-      </c>
-      <c r="C9" t="s">
-        <v>144</v>
-      </c>
-      <c r="D9" t="s">
-        <v>82</v>
-      </c>
-      <c r="E9" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A10" s="10" t="s">
-        <v>165</v>
+        <v>190</v>
       </c>
       <c r="B10" t="s">
-        <v>59</v>
+        <v>191</v>
       </c>
       <c r="C10" t="s">
         <v>139</v>
       </c>
       <c r="D10" t="s">
-        <v>73</v>
+        <v>192</v>
       </c>
       <c r="E10" t="s">
-        <v>166</v>
+        <v>193</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A11" s="10" t="s">
-        <v>167</v>
+        <v>232</v>
       </c>
       <c r="B11" t="s">
-        <v>168</v>
+        <v>86</v>
       </c>
       <c r="C11" t="s">
         <v>139</v>
       </c>
       <c r="D11" t="s">
-        <v>169</v>
+        <v>85</v>
       </c>
       <c r="E11" t="s">
-        <v>170</v>
+        <v>233</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A12" s="10" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="B12" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="C12" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="D12" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="E12" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A13" s="10" t="s">
-        <v>175</v>
+        <v>242</v>
       </c>
       <c r="B13" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C13" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="D13" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="E13" t="s">
-        <v>176</v>
+        <v>243</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A14" s="10" t="s">
-        <v>177</v>
+        <v>252</v>
       </c>
       <c r="B14" t="s">
-        <v>178</v>
+        <v>76</v>
       </c>
       <c r="C14" t="s">
         <v>139</v>
       </c>
       <c r="D14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E14" t="s">
-        <v>179</v>
+        <v>253</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A15" s="10" t="s">
-        <v>180</v>
+        <v>144</v>
       </c>
       <c r="B15" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C15" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="D15" t="s">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="E15" t="s">
-        <v>181</v>
+        <v>146</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A16" s="10" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="B16" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C16" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="D16" t="s">
-        <v>183</v>
+        <v>61</v>
       </c>
       <c r="E16" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A17" s="10" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="B17" t="s">
-        <v>186</v>
+        <v>58</v>
       </c>
       <c r="C17" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="D17" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="E17" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A18" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="B18" t="s">
+        <v>187</v>
+      </c>
+      <c r="C18" t="s">
+        <v>139</v>
+      </c>
+      <c r="D18" t="s">
+        <v>188</v>
+      </c>
+      <c r="E18" t="s">
         <v>189</v>
-      </c>
-      <c r="B18" t="s">
-        <v>190</v>
-      </c>
-      <c r="C18" t="s">
-        <v>139</v>
-      </c>
-      <c r="D18" t="s">
-        <v>191</v>
-      </c>
-      <c r="E18" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A19" s="10" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="B19" t="s">
-        <v>194</v>
+        <v>68</v>
       </c>
       <c r="C19" t="s">
         <v>139</v>
       </c>
       <c r="D19" t="s">
-        <v>195</v>
+        <v>67</v>
       </c>
       <c r="E19" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A20" s="10" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B20" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C20" t="s">
         <v>139</v>
       </c>
       <c r="D20" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="E20" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A21" s="10" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B21" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="C21" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D21" t="s">
-        <v>67</v>
+        <v>81</v>
       </c>
       <c r="E21" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A22" s="10" t="s">
-        <v>203</v>
+        <v>244</v>
       </c>
       <c r="B22" t="s">
-        <v>204</v>
+        <v>59</v>
       </c>
       <c r="C22" t="s">
         <v>139</v>
       </c>
       <c r="D22" t="s">
-        <v>205</v>
+        <v>37</v>
       </c>
       <c r="E22" t="s">
-        <v>206</v>
+        <v>245</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.4">
@@ -1789,98 +1773,98 @@
         <v>207</v>
       </c>
       <c r="B23" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="C23" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="D23" t="s">
-        <v>81</v>
+        <v>208</v>
       </c>
       <c r="E23" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A24" s="10" t="s">
-        <v>209</v>
+        <v>236</v>
       </c>
       <c r="B24" t="s">
-        <v>210</v>
+        <v>237</v>
       </c>
       <c r="C24" t="s">
         <v>139</v>
       </c>
       <c r="D24" t="s">
-        <v>211</v>
+        <v>238</v>
       </c>
       <c r="E24" t="s">
-        <v>212</v>
+        <v>239</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A25" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B25" t="s">
-        <v>72</v>
+        <v>215</v>
       </c>
       <c r="C25" t="s">
         <v>139</v>
       </c>
       <c r="D25" t="s">
-        <v>214</v>
+        <v>41</v>
       </c>
       <c r="E25" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A26" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B26" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C26" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D26" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E26" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A27" s="10" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B27" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C27" t="s">
         <v>139</v>
       </c>
       <c r="D27" t="s">
-        <v>41</v>
+        <v>223</v>
       </c>
       <c r="E27" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A28" s="10" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B28" t="s">
-        <v>224</v>
+        <v>66</v>
       </c>
       <c r="C28" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="D28" t="s">
-        <v>225</v>
+        <v>64</v>
       </c>
       <c r="E28" t="s">
         <v>226</v>
@@ -1897,248 +1881,231 @@
         <v>139</v>
       </c>
       <c r="D29" t="s">
+        <v>90</v>
+      </c>
+      <c r="E29" t="s">
         <v>229</v>
-      </c>
-      <c r="E29" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A30" s="10" t="s">
-        <v>231</v>
+        <v>168</v>
       </c>
       <c r="B30" t="s">
-        <v>66</v>
+        <v>169</v>
       </c>
       <c r="C30" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D30" t="s">
-        <v>64</v>
+        <v>170</v>
       </c>
       <c r="E30" t="s">
-        <v>232</v>
+        <v>171</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A31" s="10" t="s">
-        <v>233</v>
+        <v>258</v>
       </c>
       <c r="B31" t="s">
-        <v>234</v>
+        <v>259</v>
       </c>
       <c r="C31" t="s">
         <v>139</v>
       </c>
       <c r="D31" t="s">
-        <v>90</v>
+        <v>260</v>
       </c>
       <c r="E31" t="s">
-        <v>235</v>
+        <v>261</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A32" s="10" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="B32" t="s">
-        <v>71</v>
+        <v>262</v>
       </c>
       <c r="C32" t="s">
         <v>139</v>
       </c>
       <c r="D32" t="s">
-        <v>36</v>
+        <v>131</v>
       </c>
       <c r="E32" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A33" s="10" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="B33" t="s">
-        <v>239</v>
+        <v>206</v>
       </c>
       <c r="C33" t="s">
         <v>139</v>
       </c>
       <c r="D33" t="s">
-        <v>240</v>
+        <v>122</v>
       </c>
       <c r="E33" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A34" s="10" t="s">
-        <v>242</v>
+        <v>194</v>
       </c>
       <c r="B34" t="s">
-        <v>86</v>
+        <v>195</v>
       </c>
       <c r="C34" t="s">
         <v>139</v>
       </c>
       <c r="D34" t="s">
-        <v>85</v>
+        <v>196</v>
       </c>
       <c r="E34" t="s">
-        <v>243</v>
+        <v>197</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A35" s="10" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B35" t="s">
-        <v>210</v>
+        <v>0</v>
       </c>
       <c r="C35" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D35" t="s">
-        <v>122</v>
+        <v>1</v>
       </c>
       <c r="E35" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A36" s="10" t="s">
-        <v>246</v>
+        <v>210</v>
       </c>
       <c r="B36" t="s">
-        <v>247</v>
+        <v>211</v>
       </c>
       <c r="C36" t="s">
         <v>139</v>
       </c>
       <c r="D36" t="s">
-        <v>248</v>
+        <v>212</v>
       </c>
       <c r="E36" t="s">
-        <v>249</v>
+        <v>213</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A37" s="10" t="s">
-        <v>250</v>
+        <v>137</v>
       </c>
       <c r="B37" t="s">
-        <v>0</v>
+        <v>138</v>
       </c>
       <c r="C37" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="D37" t="s">
-        <v>1</v>
+        <v>140</v>
       </c>
       <c r="E37" t="s">
-        <v>251</v>
+        <v>141</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A38" s="10" t="s">
-        <v>252</v>
-      </c>
-      <c r="B38" t="s">
-        <v>115</v>
+        <v>174</v>
+      </c>
+      <c r="B38" s="11" t="s">
+        <v>175</v>
       </c>
       <c r="C38" t="s">
         <v>139</v>
       </c>
       <c r="D38" t="s">
-        <v>114</v>
+        <v>40</v>
       </c>
       <c r="E38" t="s">
-        <v>253</v>
+        <v>176</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A39" s="10" t="s">
-        <v>254</v>
-      </c>
-      <c r="B39" s="11" t="s">
-        <v>268</v>
+        <v>248</v>
+      </c>
+      <c r="B39" t="s">
+        <v>75</v>
       </c>
       <c r="C39" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D39" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E39" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A40" s="10" t="s">
-        <v>256</v>
+        <v>230</v>
       </c>
       <c r="B40" t="s">
-        <v>266</v>
+        <v>71</v>
       </c>
       <c r="C40" t="s">
         <v>139</v>
       </c>
       <c r="D40" t="s">
-        <v>131</v>
+        <v>36</v>
       </c>
       <c r="E40" t="s">
-        <v>257</v>
+        <v>231</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A41" s="10" t="s">
-        <v>258</v>
+        <v>142</v>
       </c>
       <c r="B41" t="s">
-        <v>75</v>
+        <v>263</v>
       </c>
       <c r="C41" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D41" t="s">
-        <v>38</v>
+        <v>250</v>
       </c>
       <c r="E41" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A42" s="10" t="s">
-        <v>142</v>
+        <v>172</v>
       </c>
       <c r="B42" t="s">
-        <v>143</v>
+        <v>116</v>
       </c>
       <c r="C42" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D42" t="s">
-        <v>260</v>
+        <v>118</v>
       </c>
       <c r="E42" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A43" s="10" t="s">
-        <v>262</v>
-      </c>
-      <c r="B43" t="s">
-        <v>76</v>
-      </c>
-      <c r="C43" t="s">
-        <v>139</v>
-      </c>
-      <c r="D43" t="s">
-        <v>39</v>
-      </c>
-      <c r="E43" t="s">
-        <v>263</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add sentence extraction support to vocab server and material uploader 2026-06-20 17:57:55
</commit_message>
<xml_diff>
--- a/服务及对应的dify文件.xlsx
+++ b/服务及对应的dify文件.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cursor\work\super-agent\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2586C9BB-1936-4FF9-836C-DA5F760496BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{027A80A3-9DAE-4CBA-8664-ADA11040F310}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" xr2:uid="{869B5D85-7F33-4AEA-A1C3-C855F7D15279}"/>
+    <workbookView xWindow="5272" yWindow="3848" windowWidth="16875" windowHeight="10432" activeTab="2" xr2:uid="{869B5D85-7F33-4AEA-A1C3-C855F7D15279}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="291">
   <si>
     <t>mychat_memory_kb</t>
   </si>
@@ -604,321 +605,385 @@
     <t>845bb27a-f65a-4521-a4d0-0323451a005e</t>
   </si>
   <si>
+    <t>app-P3RxMjvtrhr2rFAXqKcfGSFA</t>
+  </si>
+  <si>
+    <t>2026-05-0407:08:32</t>
+  </si>
+  <si>
+    <t>f4466e94-c6d8-4a3b-bf8b-0c592b45d646</t>
+  </si>
+  <si>
+    <t>2026-05-2310:04:31</t>
+  </si>
+  <si>
+    <t>262972e7-b867-4303-8ab8-795856cc844c</t>
+  </si>
+  <si>
+    <t>2026-05-1817:34:40</t>
+  </si>
+  <si>
+    <t>d7e31f94-faab-475c-89c7-58799f48e342</t>
+  </si>
+  <si>
+    <t>2026-05-1403:01:41</t>
+  </si>
+  <si>
+    <t>e04bdaa8-3d08-4439-ad67-de190ad9e557</t>
+  </si>
+  <si>
+    <t>app-UK9zXVRuldyCSGA71YQpoVpS</t>
+  </si>
+  <si>
+    <t>2026-05-1623:19:42</t>
+  </si>
+  <si>
+    <t>3f2add23-56a5-4e98-bd3d-4e8adb84cfb4</t>
+  </si>
+  <si>
+    <t>app-YTMU9kmBawVOnv9CSOandhp3</t>
+  </si>
+  <si>
+    <t>2026-05-2203:14:19</t>
+  </si>
+  <si>
+    <t>fa82503b-444f-41e7-936d-c4f8b044a337</t>
+  </si>
+  <si>
+    <t>文治系统分析引擎(WriteGovernance)</t>
+  </si>
+  <si>
+    <t>app-xcidaY4l2ZbfVwL9llFyQXKA</t>
+  </si>
+  <si>
+    <t>2026-05-2407:43:29</t>
+  </si>
+  <si>
+    <t>11470c40-9678-42a3-83f7-85cda5f02671</t>
+  </si>
+  <si>
+    <t>English_Vocab_Engine</t>
+  </si>
+  <si>
+    <t>app-bqp3Cw7pb58rOpEfDeWof6bg</t>
+  </si>
+  <si>
+    <t>2026-05-1008:49:44</t>
+  </si>
+  <si>
+    <t>0fda700d-40d1-463e-b3d3-8726cdc01d33</t>
+  </si>
+  <si>
+    <t>Memory_Aid_Engine</t>
+  </si>
+  <si>
+    <t>app-aElSukJkmKmojPkVSk6H1mmN</t>
+  </si>
+  <si>
+    <t>2026-06-0812:05:29</t>
+  </si>
+  <si>
+    <t>8ea695f9-56d2-4d51-b722-69114ea10dc3</t>
+  </si>
+  <si>
+    <t>2026-05-1304:49:20</t>
+  </si>
+  <si>
+    <t>cf33959d-92f8-4f5a-8332-329e444919ce</t>
+  </si>
+  <si>
+    <t>image2text2</t>
+  </si>
+  <si>
+    <t>app-uCbUAvW6IzHig4AOOmbRAjOZ</t>
+  </si>
+  <si>
+    <t>2026-05-0706:27:37</t>
+  </si>
+  <si>
+    <t>1f82c19d-6bf2-4622-b38a-af4438245ee9</t>
+  </si>
+  <si>
+    <t>2026-05-1906:34:23</t>
+  </si>
+  <si>
+    <t>CognitivePenetrationEngine</t>
+  </si>
+  <si>
+    <t>8d0ec4cf-384e-4a29-a628-2f7278bf843e</t>
+  </si>
+  <si>
+    <t>app-2lPI1fnTZXad15HQcF3xVZz5</t>
+  </si>
+  <si>
+    <t>2026-05-1013:10:50</t>
+  </si>
+  <si>
+    <t>3b6cf9ab-f6a6-488f-b5f6-c0edc52c3461</t>
+  </si>
+  <si>
+    <t>驭心博弈系统分析引擎(GameTheoryEngine)</t>
+  </si>
+  <si>
+    <t>app-YysFumsmeSAeJaQMobMpW24r</t>
+  </si>
+  <si>
+    <t>2026-05-2409:45:06</t>
+  </si>
+  <si>
+    <t>e6e97725-b3d6-4ae4-adb6-695027e9be62</t>
+  </si>
+  <si>
+    <t>Grammar_Polish_Engine</t>
+  </si>
+  <si>
+    <t>2026-05-1417:50:46</t>
+  </si>
+  <si>
+    <t>a7aef2c4-bdff-4404-9057-d5e53bea8073</t>
+  </si>
+  <si>
+    <t>doc_read_modiyg</t>
+  </si>
+  <si>
+    <t>app-G0wF6sc2GeDk7ZmV5l3wLtgM</t>
+  </si>
+  <si>
+    <t>2026-05-2610:57:31</t>
+  </si>
+  <si>
+    <t>d7257d88-c0c2-47d7-92dd-05d9e475ca24</t>
+  </si>
+  <si>
+    <t>listen_insett_workflow</t>
+  </si>
+  <si>
+    <t>app-NnsKzrUYKmhd89p9aC48YLzB</t>
+  </si>
+  <si>
+    <t>2026-05-2309:47:26</t>
+  </si>
+  <si>
+    <t>fff4614e-35a7-48f6-9cb7-301b9d9f3126</t>
+  </si>
+  <si>
+    <t>2026-05-1308:27:20</t>
+  </si>
+  <si>
+    <t>c3434f8f-9728-40c5-9674-4b0242be6492</t>
+  </si>
+  <si>
+    <t>power_game_matrix_workflow</t>
+  </si>
+  <si>
+    <t>2026-05-2003:27:23</t>
+  </si>
+  <si>
+    <t>e96a78a4-731f-4f96-99ea-e3ed0f9bb130</t>
+  </si>
+  <si>
+    <t>2026-05-1014:04:29</t>
+  </si>
+  <si>
+    <t>988b1ce3-1845-40f1-9211-f7b6668ec7ca</t>
+  </si>
+  <si>
+    <t>2026-04-1209:49:09</t>
+  </si>
+  <si>
+    <t>3cd2d0c7-8fcb-463f-8b3b-03f879af6539</t>
+  </si>
+  <si>
+    <t>2026-05-2406:52:28</t>
+  </si>
+  <si>
+    <t>23f90b60-7671-4130-b386-4b17b5fde233</t>
+  </si>
+  <si>
+    <t>app-sfzT1fsn8WkX5TnnIxq9qbY7</t>
+  </si>
+  <si>
+    <t>2026-05-2415:02:26</t>
+  </si>
+  <si>
+    <t>cae424a3-d1ae-4eeb-8cc5-44b1ebed3705</t>
+  </si>
+  <si>
+    <t>2026-04-1203:48:42</t>
+  </si>
+  <si>
+    <t>e2142556-f081-4425-9700-0d331dbb00d3</t>
+  </si>
+  <si>
+    <t>2026-05-2301:23:47</t>
+  </si>
+  <si>
+    <t>631a0c22-fe77-43ac-baa5-ec01211bc69e</t>
+  </si>
+  <si>
+    <t>2026-05-1417:20:13</t>
+  </si>
+  <si>
+    <t>aabd823b-7916-443e-a9f2-f357d09e2d69</t>
+  </si>
+  <si>
+    <t>2026-05-1213:53:00</t>
+  </si>
+  <si>
+    <t>f81c9849-0800-48cf-8e56-e03ef216378c</t>
+  </si>
+  <si>
+    <t>2026-05-1010:10:39</t>
+  </si>
+  <si>
+    <t>app-Eygg39qoniWss17wjWvLUvDb</t>
+  </si>
+  <si>
+    <t>2026-06-0216:15:22</t>
+  </si>
+  <si>
+    <t>2d23c873-d150-448e-9965-7e1d3094d9b1</t>
+  </si>
+  <si>
+    <t>2026-05-1007:25:00</t>
+  </si>
+  <si>
+    <t>listen_material_generator</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Listening_Comparison_Engine</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>d94f726d-d0fd-40a2-8997-3f85fd8ab3e2</t>
+  </si>
+  <si>
+    <t>app-F6daqhSXH942sBrnGki4kzZq</t>
+  </si>
+  <si>
+    <t>2026-06-0912:30:06</t>
+  </si>
+  <si>
+    <t>english_mastery_logic</t>
+  </si>
+  <si>
+    <t>694843b2-96e0-4b36-b438-c7a1110116e8</t>
+  </si>
+  <si>
+    <t>video_subtitle_transcription_workflow</t>
+  </si>
+  <si>
+    <t>app-2LpliLyJ8viBKpacvyoOHSAV</t>
+  </si>
+  <si>
+    <t>2026-06-1008:58:18</t>
+  </si>
+  <si>
+    <t>materail_generate_url_enhanced</t>
+  </si>
+  <si>
+    <t>custom_theme_extraction</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>dict_tool_workflow</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>English_Oral_Sandbox</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>English_Word_Enricher</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Impromptu_Speech_Prompter</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Insight_Listen_Engine</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>insgit_gen_flow</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AestheticEngine</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Impromptu_Speech_Exemplar</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>text2image</t>
-  </si>
-  <si>
-    <t>app-P3RxMjvtrhr2rFAXqKcfGSFA</t>
-  </si>
-  <si>
-    <t>2026-05-0407:08:32</t>
-  </si>
-  <si>
-    <t>f4466e94-c6d8-4a3b-bf8b-0c592b45d646</t>
-  </si>
-  <si>
-    <t>2026-05-2310:04:31</t>
-  </si>
-  <si>
-    <t>262972e7-b867-4303-8ab8-795856cc844c</t>
-  </si>
-  <si>
-    <t>2026-05-1817:34:40</t>
-  </si>
-  <si>
-    <t>d7e31f94-faab-475c-89c7-58799f48e342</t>
-  </si>
-  <si>
-    <t>2026-05-1403:01:41</t>
-  </si>
-  <si>
-    <t>e04bdaa8-3d08-4439-ad67-de190ad9e557</t>
-  </si>
-  <si>
-    <t>app-UK9zXVRuldyCSGA71YQpoVpS</t>
-  </si>
-  <si>
-    <t>2026-05-1623:19:42</t>
-  </si>
-  <si>
-    <t>3f2add23-56a5-4e98-bd3d-4e8adb84cfb4</t>
-  </si>
-  <si>
-    <t>app-YTMU9kmBawVOnv9CSOandhp3</t>
-  </si>
-  <si>
-    <t>2026-05-2203:14:19</t>
-  </si>
-  <si>
-    <t>fa82503b-444f-41e7-936d-c4f8b044a337</t>
-  </si>
-  <si>
-    <t>文治系统分析引擎(WriteGovernance)</t>
-  </si>
-  <si>
-    <t>app-xcidaY4l2ZbfVwL9llFyQXKA</t>
-  </si>
-  <si>
-    <t>2026-05-2407:43:29</t>
-  </si>
-  <si>
-    <t>11470c40-9678-42a3-83f7-85cda5f02671</t>
-  </si>
-  <si>
-    <t>English_Vocab_Engine</t>
-  </si>
-  <si>
-    <t>app-bqp3Cw7pb58rOpEfDeWof6bg</t>
-  </si>
-  <si>
-    <t>2026-05-1008:49:44</t>
-  </si>
-  <si>
-    <t>0fda700d-40d1-463e-b3d3-8726cdc01d33</t>
-  </si>
-  <si>
-    <t>Memory_Aid_Engine</t>
-  </si>
-  <si>
-    <t>app-aElSukJkmKmojPkVSk6H1mmN</t>
-  </si>
-  <si>
-    <t>2026-06-0812:05:29</t>
-  </si>
-  <si>
-    <t>8ea695f9-56d2-4d51-b722-69114ea10dc3</t>
-  </si>
-  <si>
-    <t>2026-05-1304:49:20</t>
-  </si>
-  <si>
-    <t>cf33959d-92f8-4f5a-8332-329e444919ce</t>
-  </si>
-  <si>
-    <t>image2text2</t>
-  </si>
-  <si>
-    <t>app-uCbUAvW6IzHig4AOOmbRAjOZ</t>
-  </si>
-  <si>
-    <t>2026-05-0706:27:37</t>
-  </si>
-  <si>
-    <t>1f82c19d-6bf2-4622-b38a-af4438245ee9</t>
-  </si>
-  <si>
-    <t>2026-05-1906:34:23</t>
-  </si>
-  <si>
-    <t>CognitivePenetrationEngine</t>
-  </si>
-  <si>
-    <t>8d0ec4cf-384e-4a29-a628-2f7278bf843e</t>
-  </si>
-  <si>
-    <t>app-2lPI1fnTZXad15HQcF3xVZz5</t>
-  </si>
-  <si>
-    <t>2026-05-1013:10:50</t>
-  </si>
-  <si>
-    <t>3b6cf9ab-f6a6-488f-b5f6-c0edc52c3461</t>
-  </si>
-  <si>
-    <t>驭心博弈系统分析引擎(GameTheoryEngine)</t>
-  </si>
-  <si>
-    <t>app-YysFumsmeSAeJaQMobMpW24r</t>
-  </si>
-  <si>
-    <t>2026-05-2409:45:06</t>
-  </si>
-  <si>
-    <t>e6e97725-b3d6-4ae4-adb6-695027e9be62</t>
-  </si>
-  <si>
-    <t>Grammar_Polish_Engine</t>
-  </si>
-  <si>
-    <t>2026-05-1417:50:46</t>
-  </si>
-  <si>
-    <t>a7aef2c4-bdff-4404-9057-d5e53bea8073</t>
-  </si>
-  <si>
-    <t>doc_read_modiyg</t>
-  </si>
-  <si>
-    <t>app-G0wF6sc2GeDk7ZmV5l3wLtgM</t>
-  </si>
-  <si>
-    <t>2026-05-2610:57:31</t>
-  </si>
-  <si>
-    <t>d7257d88-c0c2-47d7-92dd-05d9e475ca24</t>
-  </si>
-  <si>
-    <t>listen_insett_workflow</t>
-  </si>
-  <si>
-    <t>app-NnsKzrUYKmhd89p9aC48YLzB</t>
-  </si>
-  <si>
-    <t>2026-05-2309:47:26</t>
-  </si>
-  <si>
-    <t>fff4614e-35a7-48f6-9cb7-301b9d9f3126</t>
-  </si>
-  <si>
-    <t>2026-05-1308:27:20</t>
-  </si>
-  <si>
-    <t>c3434f8f-9728-40c5-9674-4b0242be6492</t>
-  </si>
-  <si>
-    <t>power_game_matrix_workflow</t>
-  </si>
-  <si>
-    <t>2026-05-2003:27:23</t>
-  </si>
-  <si>
-    <t>e96a78a4-731f-4f96-99ea-e3ed0f9bb130</t>
-  </si>
-  <si>
-    <t>2026-05-1014:04:29</t>
-  </si>
-  <si>
-    <t>988b1ce3-1845-40f1-9211-f7b6668ec7ca</t>
-  </si>
-  <si>
-    <t>2026-04-1209:49:09</t>
-  </si>
-  <si>
-    <t>3cd2d0c7-8fcb-463f-8b3b-03f879af6539</t>
-  </si>
-  <si>
-    <t>2026-05-2406:52:28</t>
-  </si>
-  <si>
-    <t>23f90b60-7671-4130-b386-4b17b5fde233</t>
-  </si>
-  <si>
-    <t>app-sfzT1fsn8WkX5TnnIxq9qbY7</t>
-  </si>
-  <si>
-    <t>2026-05-2415:02:26</t>
-  </si>
-  <si>
-    <t>cae424a3-d1ae-4eeb-8cc5-44b1ebed3705</t>
-  </si>
-  <si>
-    <t>2026-04-1203:48:42</t>
-  </si>
-  <si>
-    <t>e2142556-f081-4425-9700-0d331dbb00d3</t>
-  </si>
-  <si>
-    <t>2026-05-2301:23:47</t>
-  </si>
-  <si>
-    <t>631a0c22-fe77-43ac-baa5-ec01211bc69e</t>
-  </si>
-  <si>
-    <t>2026-05-1417:20:13</t>
-  </si>
-  <si>
-    <t>aabd823b-7916-443e-a9f2-f357d09e2d69</t>
-  </si>
-  <si>
-    <t>2026-05-1213:53:00</t>
-  </si>
-  <si>
-    <t>f81c9849-0800-48cf-8e56-e03ef216378c</t>
-  </si>
-  <si>
-    <t>2026-05-1010:10:39</t>
-  </si>
-  <si>
-    <t>app-Eygg39qoniWss17wjWvLUvDb</t>
-  </si>
-  <si>
-    <t>2026-06-0216:15:22</t>
-  </si>
-  <si>
-    <t>2d23c873-d150-448e-9965-7e1d3094d9b1</t>
-  </si>
-  <si>
-    <t>2026-05-1007:25:00</t>
-  </si>
-  <si>
-    <t>listen_material_generator</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Listening_Comparison_Engine</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>d94f726d-d0fd-40a2-8997-3f85fd8ab3e2</t>
-  </si>
-  <si>
-    <t>app-F6daqhSXH942sBrnGki4kzZq</t>
-  </si>
-  <si>
-    <t>2026-06-0912:30:06</t>
-  </si>
-  <si>
-    <t>english_mastery_logic</t>
-  </si>
-  <si>
-    <t>694843b2-96e0-4b36-b438-c7a1110116e8</t>
-  </si>
-  <si>
-    <t>video_subtitle_transcription_workflow</t>
-  </si>
-  <si>
-    <t>app-2LpliLyJ8viBKpacvyoOHSAV</t>
-  </si>
-  <si>
-    <t>2026-06-1008:58:18</t>
-  </si>
-  <si>
-    <t>materail_generate_url_enhanced</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Impromptu_Speech_Prompter</t>
+  </si>
+  <si>
+    <t>06744f55-096b-43b6-946a-4ed48f9c4902</t>
+  </si>
+  <si>
+    <t>Speak_Influence_Engine</t>
+  </si>
+  <si>
+    <t>app-33cYBQOXUKbRJkurDVGkzeUS</t>
+  </si>
+  <si>
+    <t>2026-05-2310:29:35</t>
+  </si>
+  <si>
+    <t>text2image</t>
+  </si>
+  <si>
+    <t>f76f76e0-aeee-4aee-9357-9626c45b34d9</t>
+  </si>
+  <si>
+    <t>app-ZWGbI5uCdKFXj9B2yCD0Z86d</t>
+  </si>
+  <si>
+    <t>2026-05-2407:27:16</t>
+  </si>
+  <si>
+    <t>6ef856c5-a31e-466a-8c8d-35913a102eec</t>
+  </si>
+  <si>
+    <t>CognitiveAscensionEngine</t>
+  </si>
+  <si>
+    <t>app-r2UBg87br895ssEcjNhXY4je</t>
+  </si>
+  <si>
+    <t>2026-06-1316:13:15</t>
+  </si>
+  <si>
+    <t>app-OShKY1EcVuLFkuxrpO28ZB0A</t>
+  </si>
+  <si>
+    <t>2026-06-0710:52:33</t>
   </si>
   <si>
     <t>custom_theme_extraction</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>dict_tool_workflow</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>English_Oral_Sandbox</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>English_Word_Enricher</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Impromptu_Speech_Prompter</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Insight_Listen_Engine</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>insgit_gen_flow</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>AestheticEngine</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>english_wakeup_routine</t>
   </si>
   <si>
     <t>Impromptu_Speech_Exemplar</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Impromptu_Speech_Evaluation</t>
+  </si>
+  <si>
+    <t>(45rows)</t>
   </si>
 </sst>
 </file>
@@ -1438,19 +1503,19 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A2" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="B2" t="s">
+        <v>264</v>
+      </c>
+      <c r="C2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D2" t="s">
         <v>180</v>
       </c>
-      <c r="B2" t="s">
-        <v>265</v>
-      </c>
-      <c r="C2" t="s">
-        <v>138</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>181</v>
-      </c>
-      <c r="E2" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.4">
@@ -1506,19 +1571,19 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A6" s="10" t="s">
+        <v>251</v>
+      </c>
+      <c r="B6" t="s">
+        <v>260</v>
+      </c>
+      <c r="C6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D6" t="s">
         <v>252</v>
       </c>
-      <c r="B6" t="s">
-        <v>261</v>
-      </c>
-      <c r="C6" t="s">
-        <v>138</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>253</v>
-      </c>
-      <c r="E6" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.4">
@@ -1526,7 +1591,7 @@
         <v>149</v>
       </c>
       <c r="B7" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C7" t="s">
         <v>138</v>
@@ -1574,27 +1639,27 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A10" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="B10" t="s">
         <v>187</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
+        <v>138</v>
+      </c>
+      <c r="D10" t="s">
         <v>188</v>
       </c>
-      <c r="C10" t="s">
-        <v>138</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>189</v>
-      </c>
-      <c r="E10" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A11" s="10" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B11" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C11" t="s">
         <v>138</v>
@@ -1603,7 +1668,7 @@
         <v>85</v>
       </c>
       <c r="E11" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.4">
@@ -1625,10 +1690,10 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A13" s="10" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B13" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C13" t="s">
         <v>138</v>
@@ -1637,12 +1702,12 @@
         <v>114</v>
       </c>
       <c r="E13" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A14" s="10" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B14" t="s">
         <v>76</v>
@@ -1654,7 +1719,7 @@
         <v>39</v>
       </c>
       <c r="E14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.4">
@@ -1662,7 +1727,7 @@
         <v>143</v>
       </c>
       <c r="B15" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C15" t="s">
         <v>144</v>
@@ -1676,7 +1741,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A16" s="10" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B16" t="s">
         <v>62</v>
@@ -1688,12 +1753,12 @@
         <v>61</v>
       </c>
       <c r="E16" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A17" s="10" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B17" t="s">
         <v>58</v>
@@ -1702,32 +1767,32 @@
         <v>144</v>
       </c>
       <c r="D17" t="s">
+        <v>177</v>
+      </c>
+      <c r="E17" t="s">
         <v>178</v>
-      </c>
-      <c r="E17" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A18" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="B18" t="s">
         <v>183</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
+        <v>138</v>
+      </c>
+      <c r="D18" t="s">
         <v>184</v>
       </c>
-      <c r="C18" t="s">
-        <v>138</v>
-      </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>185</v>
-      </c>
-      <c r="E18" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A19" s="10" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B19" t="s">
         <v>68</v>
@@ -1739,29 +1804,29 @@
         <v>67</v>
       </c>
       <c r="E19" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A20" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="B20" t="s">
         <v>197</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
+        <v>138</v>
+      </c>
+      <c r="D20" t="s">
         <v>198</v>
       </c>
-      <c r="C20" t="s">
-        <v>138</v>
-      </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>199</v>
-      </c>
-      <c r="E20" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A21" s="10" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B21" t="s">
         <v>79</v>
@@ -1773,15 +1838,15 @@
         <v>81</v>
       </c>
       <c r="E21" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A22" s="10" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B22" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C22" t="s">
         <v>138</v>
@@ -1790,12 +1855,12 @@
         <v>37</v>
       </c>
       <c r="E22" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A23" s="10" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B23" t="s">
         <v>72</v>
@@ -1804,35 +1869,35 @@
         <v>138</v>
       </c>
       <c r="D23" t="s">
+        <v>204</v>
+      </c>
+      <c r="E23" t="s">
         <v>205</v>
-      </c>
-      <c r="E23" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A24" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="B24" t="s">
+        <v>267</v>
+      </c>
+      <c r="C24" t="s">
+        <v>138</v>
+      </c>
+      <c r="D24" t="s">
         <v>233</v>
       </c>
-      <c r="B24" t="s">
-        <v>268</v>
-      </c>
-      <c r="C24" t="s">
-        <v>138</v>
-      </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
         <v>234</v>
-      </c>
-      <c r="E24" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A25" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="B25" t="s">
         <v>211</v>
-      </c>
-      <c r="B25" t="s">
-        <v>212</v>
       </c>
       <c r="C25" t="s">
         <v>138</v>
@@ -1841,46 +1906,46 @@
         <v>41</v>
       </c>
       <c r="E25" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A26" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="B26" t="s">
         <v>214</v>
-      </c>
-      <c r="B26" t="s">
-        <v>215</v>
       </c>
       <c r="C26" t="s">
         <v>142</v>
       </c>
       <c r="D26" t="s">
+        <v>215</v>
+      </c>
+      <c r="E26" t="s">
         <v>216</v>
-      </c>
-      <c r="E26" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A27" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="B27" t="s">
         <v>218</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C27" t="s">
+        <v>138</v>
+      </c>
+      <c r="D27" t="s">
         <v>219</v>
       </c>
-      <c r="C27" t="s">
-        <v>138</v>
-      </c>
-      <c r="D27" t="s">
+      <c r="E27" t="s">
         <v>220</v>
-      </c>
-      <c r="E27" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A28" s="10" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B28" t="s">
         <v>66</v>
@@ -1892,15 +1957,15 @@
         <v>64</v>
       </c>
       <c r="E28" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A29" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="B29" t="s">
         <v>224</v>
-      </c>
-      <c r="B29" t="s">
-        <v>225</v>
       </c>
       <c r="C29" t="s">
         <v>138</v>
@@ -1909,7 +1974,7 @@
         <v>90</v>
       </c>
       <c r="E29" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.4">
@@ -1917,38 +1982,38 @@
         <v>167</v>
       </c>
       <c r="B30" t="s">
-        <v>168</v>
+        <v>269</v>
       </c>
       <c r="C30" t="s">
         <v>142</v>
       </c>
       <c r="D30" t="s">
+        <v>168</v>
+      </c>
+      <c r="E30" t="s">
         <v>169</v>
-      </c>
-      <c r="E30" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A31" s="10" t="s">
+        <v>255</v>
+      </c>
+      <c r="B31" t="s">
         <v>256</v>
       </c>
-      <c r="B31" t="s">
+      <c r="C31" t="s">
+        <v>138</v>
+      </c>
+      <c r="D31" t="s">
         <v>257</v>
       </c>
-      <c r="C31" t="s">
-        <v>138</v>
-      </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>258</v>
-      </c>
-      <c r="E31" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A32" s="10" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B32" t="s">
         <v>130</v>
@@ -1960,15 +2025,15 @@
         <v>131</v>
       </c>
       <c r="E32" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A33" s="10" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B33" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C33" t="s">
         <v>138</v>
@@ -1977,29 +2042,29 @@
         <v>122</v>
       </c>
       <c r="E33" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A34" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="B34" t="s">
         <v>191</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
+        <v>138</v>
+      </c>
+      <c r="D34" t="s">
         <v>192</v>
       </c>
-      <c r="C34" t="s">
-        <v>138</v>
-      </c>
-      <c r="D34" t="s">
+      <c r="E34" t="s">
         <v>193</v>
-      </c>
-      <c r="E34" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A35" s="10" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B35" t="s">
         <v>0</v>
@@ -2011,24 +2076,24 @@
         <v>1</v>
       </c>
       <c r="E35" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A36" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="B36" t="s">
         <v>207</v>
       </c>
-      <c r="B36" t="s">
+      <c r="C36" t="s">
+        <v>138</v>
+      </c>
+      <c r="D36" t="s">
         <v>208</v>
       </c>
-      <c r="C36" t="s">
-        <v>138</v>
-      </c>
-      <c r="D36" t="s">
+      <c r="E36" t="s">
         <v>209</v>
-      </c>
-      <c r="E36" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.4">
@@ -2036,7 +2101,7 @@
         <v>137</v>
       </c>
       <c r="B37" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C37" t="s">
         <v>138</v>
@@ -2050,7 +2115,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A38" s="10" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B38" s="11" t="s">
         <v>113</v>
@@ -2062,15 +2127,15 @@
         <v>40</v>
       </c>
       <c r="E38" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A39" s="10" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B39" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C39" t="s">
         <v>142</v>
@@ -2079,15 +2144,15 @@
         <v>38</v>
       </c>
       <c r="E39" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A40" s="10" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B40" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C40" t="s">
         <v>138</v>
@@ -2096,7 +2161,7 @@
         <v>36</v>
       </c>
       <c r="E40" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.4">
@@ -2104,24 +2169,24 @@
         <v>141</v>
       </c>
       <c r="B41" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C41" t="s">
         <v>142</v>
       </c>
       <c r="D41" t="s">
+        <v>245</v>
+      </c>
+      <c r="E41" t="s">
         <v>246</v>
-      </c>
-      <c r="E41" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A42" s="10" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B42" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C42" t="s">
         <v>144</v>
@@ -2130,7 +2195,7 @@
         <v>118</v>
       </c>
       <c r="E42" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -2660,4 +2725,807 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE5AECD3-6EB5-448C-B53F-1C3E6E1A6604}">
+  <dimension ref="A1:E47"/>
+  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="40.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.46484375" customWidth="1"/>
+    <col min="4" max="4" width="34" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A1" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="B1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C1" t="s">
+        <v>134</v>
+      </c>
+      <c r="D1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A2" t="s">
+        <v>179</v>
+      </c>
+      <c r="B2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D2" t="s">
+        <v>180</v>
+      </c>
+      <c r="E2" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A3" t="s">
+        <v>149</v>
+      </c>
+      <c r="B3" t="s">
+        <v>254</v>
+      </c>
+      <c r="C3" t="s">
+        <v>138</v>
+      </c>
+      <c r="D3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B4" t="s">
+        <v>147</v>
+      </c>
+      <c r="C4" t="s">
+        <v>138</v>
+      </c>
+      <c r="D4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E4" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A5" t="s">
+        <v>210</v>
+      </c>
+      <c r="B5" t="s">
+        <v>211</v>
+      </c>
+      <c r="C5" t="s">
+        <v>138</v>
+      </c>
+      <c r="D5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E5" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A6" t="s">
+        <v>155</v>
+      </c>
+      <c r="B6" t="s">
+        <v>156</v>
+      </c>
+      <c r="C6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D6" t="s">
+        <v>157</v>
+      </c>
+      <c r="E6" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A7" t="s">
+        <v>159</v>
+      </c>
+      <c r="B7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7" t="s">
+        <v>142</v>
+      </c>
+      <c r="D7" t="s">
+        <v>82</v>
+      </c>
+      <c r="E7" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A8" t="s">
+        <v>161</v>
+      </c>
+      <c r="B8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C8" t="s">
+        <v>138</v>
+      </c>
+      <c r="D8" t="s">
+        <v>73</v>
+      </c>
+      <c r="E8" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A9" t="s">
+        <v>239</v>
+      </c>
+      <c r="B9" t="s">
+        <v>59</v>
+      </c>
+      <c r="C9" t="s">
+        <v>138</v>
+      </c>
+      <c r="D9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A10" t="s">
+        <v>163</v>
+      </c>
+      <c r="B10" t="s">
+        <v>164</v>
+      </c>
+      <c r="C10" t="s">
+        <v>138</v>
+      </c>
+      <c r="D10" t="s">
+        <v>165</v>
+      </c>
+      <c r="E10" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A11" t="s">
+        <v>237</v>
+      </c>
+      <c r="B11" t="s">
+        <v>115</v>
+      </c>
+      <c r="C11" t="s">
+        <v>138</v>
+      </c>
+      <c r="D11" t="s">
+        <v>114</v>
+      </c>
+      <c r="E11" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A12" t="s">
+        <v>271</v>
+      </c>
+      <c r="B12" t="s">
+        <v>272</v>
+      </c>
+      <c r="C12" t="s">
+        <v>138</v>
+      </c>
+      <c r="D12" t="s">
+        <v>273</v>
+      </c>
+      <c r="E12" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A13" t="s">
+        <v>167</v>
+      </c>
+      <c r="B13" t="s">
+        <v>275</v>
+      </c>
+      <c r="C13" t="s">
+        <v>142</v>
+      </c>
+      <c r="D13" t="s">
+        <v>168</v>
+      </c>
+      <c r="E13" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A14" t="s">
+        <v>174</v>
+      </c>
+      <c r="B14" t="s">
+        <v>62</v>
+      </c>
+      <c r="C14" t="s">
+        <v>138</v>
+      </c>
+      <c r="D14" t="s">
+        <v>61</v>
+      </c>
+      <c r="E14" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A15" t="s">
+        <v>176</v>
+      </c>
+      <c r="B15" t="s">
+        <v>58</v>
+      </c>
+      <c r="C15" t="s">
+        <v>144</v>
+      </c>
+      <c r="D15" t="s">
+        <v>177</v>
+      </c>
+      <c r="E15" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A16" t="s">
+        <v>182</v>
+      </c>
+      <c r="B16" t="s">
+        <v>183</v>
+      </c>
+      <c r="C16" t="s">
+        <v>138</v>
+      </c>
+      <c r="D16" t="s">
+        <v>184</v>
+      </c>
+      <c r="E16" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A17" t="s">
+        <v>206</v>
+      </c>
+      <c r="B17" t="s">
+        <v>207</v>
+      </c>
+      <c r="C17" t="s">
+        <v>138</v>
+      </c>
+      <c r="D17" t="s">
+        <v>208</v>
+      </c>
+      <c r="E17" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A18" t="s">
+        <v>194</v>
+      </c>
+      <c r="B18" t="s">
+        <v>68</v>
+      </c>
+      <c r="C18" t="s">
+        <v>138</v>
+      </c>
+      <c r="D18" t="s">
+        <v>67</v>
+      </c>
+      <c r="E18" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A19" t="s">
+        <v>196</v>
+      </c>
+      <c r="B19" t="s">
+        <v>197</v>
+      </c>
+      <c r="C19" t="s">
+        <v>138</v>
+      </c>
+      <c r="D19" t="s">
+        <v>198</v>
+      </c>
+      <c r="E19" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A20" t="s">
+        <v>200</v>
+      </c>
+      <c r="B20" t="s">
+        <v>79</v>
+      </c>
+      <c r="C20" t="s">
+        <v>142</v>
+      </c>
+      <c r="D20" t="s">
+        <v>81</v>
+      </c>
+      <c r="E20" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A21" t="s">
+        <v>170</v>
+      </c>
+      <c r="B21" t="s">
+        <v>116</v>
+      </c>
+      <c r="C21" t="s">
+        <v>144</v>
+      </c>
+      <c r="D21" t="s">
+        <v>118</v>
+      </c>
+      <c r="E21" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A22" t="s">
+        <v>243</v>
+      </c>
+      <c r="B22" t="s">
+        <v>75</v>
+      </c>
+      <c r="C22" t="s">
+        <v>142</v>
+      </c>
+      <c r="D22" t="s">
+        <v>38</v>
+      </c>
+      <c r="E22" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A23" t="s">
+        <v>213</v>
+      </c>
+      <c r="B23" t="s">
+        <v>214</v>
+      </c>
+      <c r="C23" t="s">
+        <v>142</v>
+      </c>
+      <c r="D23" t="s">
+        <v>215</v>
+      </c>
+      <c r="E23" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A24" t="s">
+        <v>217</v>
+      </c>
+      <c r="B24" t="s">
+        <v>218</v>
+      </c>
+      <c r="C24" t="s">
+        <v>138</v>
+      </c>
+      <c r="D24" t="s">
+        <v>219</v>
+      </c>
+      <c r="E24" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A25" t="s">
+        <v>221</v>
+      </c>
+      <c r="B25" t="s">
+        <v>66</v>
+      </c>
+      <c r="C25" t="s">
+        <v>138</v>
+      </c>
+      <c r="D25" t="s">
+        <v>64</v>
+      </c>
+      <c r="E25" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A26" t="s">
+        <v>223</v>
+      </c>
+      <c r="B26" t="s">
+        <v>224</v>
+      </c>
+      <c r="C26" t="s">
+        <v>138</v>
+      </c>
+      <c r="D26" t="s">
+        <v>90</v>
+      </c>
+      <c r="E26" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A27" t="s">
+        <v>276</v>
+      </c>
+      <c r="B27" t="s">
+        <v>202</v>
+      </c>
+      <c r="C27" t="s">
+        <v>138</v>
+      </c>
+      <c r="D27" t="s">
+        <v>277</v>
+      </c>
+      <c r="E27" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A28" t="s">
+        <v>279</v>
+      </c>
+      <c r="B28" t="s">
+        <v>280</v>
+      </c>
+      <c r="C28" t="s">
+        <v>138</v>
+      </c>
+      <c r="D28" t="s">
+        <v>281</v>
+      </c>
+      <c r="E28" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A29" t="s">
+        <v>141</v>
+      </c>
+      <c r="B29" t="s">
+        <v>259</v>
+      </c>
+      <c r="C29" t="s">
+        <v>142</v>
+      </c>
+      <c r="D29" t="s">
+        <v>283</v>
+      </c>
+      <c r="E29" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A30" t="s">
+        <v>255</v>
+      </c>
+      <c r="B30" t="s">
+        <v>256</v>
+      </c>
+      <c r="C30" t="s">
+        <v>138</v>
+      </c>
+      <c r="D30" t="s">
+        <v>257</v>
+      </c>
+      <c r="E30" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A31" t="s">
+        <v>251</v>
+      </c>
+      <c r="B31" t="s">
+        <v>285</v>
+      </c>
+      <c r="C31" t="s">
+        <v>138</v>
+      </c>
+      <c r="D31" t="s">
+        <v>252</v>
+      </c>
+      <c r="E31" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A32" t="s">
+        <v>230</v>
+      </c>
+      <c r="B32" t="s">
+        <v>202</v>
+      </c>
+      <c r="C32" t="s">
+        <v>138</v>
+      </c>
+      <c r="D32" t="s">
+        <v>122</v>
+      </c>
+      <c r="E32" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A33" t="s">
+        <v>232</v>
+      </c>
+      <c r="B33" t="s">
+        <v>286</v>
+      </c>
+      <c r="C33" t="s">
+        <v>138</v>
+      </c>
+      <c r="D33" t="s">
+        <v>233</v>
+      </c>
+      <c r="E33" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A34" t="s">
+        <v>190</v>
+      </c>
+      <c r="B34" t="s">
+        <v>191</v>
+      </c>
+      <c r="C34" t="s">
+        <v>138</v>
+      </c>
+      <c r="D34" t="s">
+        <v>192</v>
+      </c>
+      <c r="E34" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A35" t="s">
+        <v>143</v>
+      </c>
+      <c r="B35" t="s">
+        <v>58</v>
+      </c>
+      <c r="C35" t="s">
+        <v>144</v>
+      </c>
+      <c r="D35" t="s">
+        <v>35</v>
+      </c>
+      <c r="E35" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A36" t="s">
+        <v>235</v>
+      </c>
+      <c r="B36" t="s">
+        <v>0</v>
+      </c>
+      <c r="C36" t="s">
+        <v>142</v>
+      </c>
+      <c r="D36" t="s">
+        <v>1</v>
+      </c>
+      <c r="E36" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A37" t="s">
+        <v>241</v>
+      </c>
+      <c r="B37" t="s">
+        <v>287</v>
+      </c>
+      <c r="C37" t="s">
+        <v>138</v>
+      </c>
+      <c r="D37" t="s">
+        <v>131</v>
+      </c>
+      <c r="E37" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A38" t="s">
+        <v>137</v>
+      </c>
+      <c r="B38" t="s">
+        <v>288</v>
+      </c>
+      <c r="C38" t="s">
+        <v>138</v>
+      </c>
+      <c r="D38" t="s">
+        <v>139</v>
+      </c>
+      <c r="E38" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A39" t="s">
+        <v>172</v>
+      </c>
+      <c r="B39" t="s">
+        <v>289</v>
+      </c>
+      <c r="C39" t="s">
+        <v>138</v>
+      </c>
+      <c r="D39" t="s">
+        <v>40</v>
+      </c>
+      <c r="E39" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A40" t="s">
+        <v>151</v>
+      </c>
+      <c r="B40" t="s">
+        <v>152</v>
+      </c>
+      <c r="C40" t="s">
+        <v>138</v>
+      </c>
+      <c r="D40" t="s">
+        <v>153</v>
+      </c>
+      <c r="E40" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A41" t="s">
+        <v>228</v>
+      </c>
+      <c r="B41" t="s">
+        <v>86</v>
+      </c>
+      <c r="C41" t="s">
+        <v>138</v>
+      </c>
+      <c r="D41" t="s">
+        <v>85</v>
+      </c>
+      <c r="E41" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A42" t="s">
+        <v>186</v>
+      </c>
+      <c r="B42" t="s">
+        <v>187</v>
+      </c>
+      <c r="C42" t="s">
+        <v>138</v>
+      </c>
+      <c r="D42" t="s">
+        <v>188</v>
+      </c>
+      <c r="E42" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A43" t="s">
+        <v>141</v>
+      </c>
+      <c r="B43" t="s">
+        <v>259</v>
+      </c>
+      <c r="C43" t="s">
+        <v>142</v>
+      </c>
+      <c r="D43" t="s">
+        <v>245</v>
+      </c>
+      <c r="E43" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A44" t="s">
+        <v>226</v>
+      </c>
+      <c r="B44" t="s">
+        <v>71</v>
+      </c>
+      <c r="C44" t="s">
+        <v>138</v>
+      </c>
+      <c r="D44" t="s">
+        <v>36</v>
+      </c>
+      <c r="E44" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A45" t="s">
+        <v>203</v>
+      </c>
+      <c r="B45" t="s">
+        <v>72</v>
+      </c>
+      <c r="C45" t="s">
+        <v>138</v>
+      </c>
+      <c r="D45" t="s">
+        <v>204</v>
+      </c>
+      <c r="E45" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A46" t="s">
+        <v>247</v>
+      </c>
+      <c r="B46" t="s">
+        <v>76</v>
+      </c>
+      <c r="C46" t="s">
+        <v>138</v>
+      </c>
+      <c r="D46" t="s">
+        <v>39</v>
+      </c>
+      <c r="E46" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A47" t="s">
+        <v>290</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>